<commit_message>
Aggiornamento automatico del sito — 16/09/2026 12:20
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3E5617-8C1A-4865-99F2-B8F56F7C1ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424C8256-A2BE-41BF-87BC-91C5A403DACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="460">
   <si>
     <t>ID</t>
   </si>
@@ -1387,6 +1387,21 @@
   </si>
   <si>
     <t>https://archive.org/details/avanziamo-lungo-la-via/mode/2up</t>
+  </si>
+  <si>
+    <t>AMI-0093</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/ai-comunisti-ai-lavoratori/mode/2up</t>
+  </si>
+  <si>
+    <t>Firenze</t>
+  </si>
+  <si>
+    <t>Centro Karl Marx</t>
+  </si>
+  <si>
+    <t>Ai comunisti ai lavoratori</t>
   </si>
 </sst>
 </file>
@@ -1446,7 +1461,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1456,6 +1471,7 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1812,7 +1828,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P93"/>
+  <dimension ref="A1:P94"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" customWidth="1"/>
@@ -5018,6 +5034,38 @@
       </c>
       <c r="M93" s="3" t="s">
         <v>454</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>455</v>
+      </c>
+      <c r="B94" t="s">
+        <v>459</v>
+      </c>
+      <c r="C94" t="s">
+        <v>458</v>
+      </c>
+      <c r="D94" t="s">
+        <v>458</v>
+      </c>
+      <c r="F94" s="9">
+        <v>26085</v>
+      </c>
+      <c r="G94" t="s">
+        <v>26</v>
+      </c>
+      <c r="H94" t="s">
+        <v>457</v>
+      </c>
+      <c r="I94" t="s">
+        <v>68</v>
+      </c>
+      <c r="L94" t="s">
+        <v>314</v>
+      </c>
+      <c r="M94" s="3" t="s">
+        <v>456</v>
       </c>
     </row>
   </sheetData>
@@ -5115,10 +5163,11 @@
     <hyperlink ref="M91" r:id="rId90" xr:uid="{734F4C0D-ECE0-4D17-AED2-596C8405BA52}"/>
     <hyperlink ref="M70" r:id="rId91" xr:uid="{410C497E-B7A6-4A52-BDB5-CD7FDB43C527}"/>
     <hyperlink ref="M93" r:id="rId92" xr:uid="{A1560D73-B423-4F16-8BB5-470F2068279E}"/>
+    <hyperlink ref="M94" r:id="rId93" xr:uid="{5C1389EE-7B8E-4CE1-AD67-A06B346AE661}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId93"/>
+    <tablePart r:id="rId94"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 19/09/2026 16:55
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424C8256-A2BE-41BF-87BC-91C5A403DACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BABC0C2-4D01-402A-A898-792DA291A622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="467">
   <si>
     <t>ID</t>
   </si>
@@ -1402,6 +1402,27 @@
   </si>
   <si>
     <t>Ai comunisti ai lavoratori</t>
+  </si>
+  <si>
+    <t>06/1971</t>
+  </si>
+  <si>
+    <t>AMI-0094</t>
+  </si>
+  <si>
+    <t>AMI-0095</t>
+  </si>
+  <si>
+    <t>Contro il liberalismo</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1968-contro-il-liberalismo/mode/2up</t>
+  </si>
+  <si>
+    <t>Presentazione della rivista Il Comunista</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/1969-presentazione-il-comunista/mode/2up</t>
   </si>
 </sst>
 </file>
@@ -1461,7 +1482,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1471,7 +1492,6 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1828,7 +1848,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P94"/>
+  <dimension ref="A1:P96"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" customWidth="1"/>
@@ -5049,8 +5069,8 @@
       <c r="D94" t="s">
         <v>458</v>
       </c>
-      <c r="F94" s="9">
-        <v>26085</v>
+      <c r="F94" s="5" t="s">
+        <v>460</v>
       </c>
       <c r="G94" t="s">
         <v>26</v>
@@ -5066,6 +5086,79 @@
       </c>
       <c r="M94" s="3" t="s">
         <v>456</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>461</v>
+      </c>
+      <c r="B95" t="s">
+        <v>463</v>
+      </c>
+      <c r="C95" t="s">
+        <v>17</v>
+      </c>
+      <c r="D95" t="s">
+        <v>18</v>
+      </c>
+      <c r="E95" t="s">
+        <v>19</v>
+      </c>
+      <c r="F95">
+        <v>1968</v>
+      </c>
+      <c r="G95" t="s">
+        <v>26</v>
+      </c>
+      <c r="H95" t="s">
+        <v>21</v>
+      </c>
+      <c r="I95" t="s">
+        <v>34</v>
+      </c>
+      <c r="L95" t="s">
+        <v>313</v>
+      </c>
+      <c r="M95" s="3" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>462</v>
+      </c>
+      <c r="B96" t="s">
+        <v>465</v>
+      </c>
+      <c r="C96" t="s">
+        <v>17</v>
+      </c>
+      <c r="D96" t="s">
+        <v>18</v>
+      </c>
+      <c r="E96" t="s">
+        <v>19</v>
+      </c>
+      <c r="F96">
+        <v>1969</v>
+      </c>
+      <c r="G96" t="s">
+        <v>26</v>
+      </c>
+      <c r="H96" t="s">
+        <v>21</v>
+      </c>
+      <c r="I96" t="s">
+        <v>34</v>
+      </c>
+      <c r="K96" t="s">
+        <v>196</v>
+      </c>
+      <c r="L96" t="s">
+        <v>313</v>
+      </c>
+      <c r="M96" s="3" t="s">
+        <v>466</v>
       </c>
     </row>
   </sheetData>
@@ -5164,10 +5257,12 @@
     <hyperlink ref="M70" r:id="rId91" xr:uid="{410C497E-B7A6-4A52-BDB5-CD7FDB43C527}"/>
     <hyperlink ref="M93" r:id="rId92" xr:uid="{A1560D73-B423-4F16-8BB5-470F2068279E}"/>
     <hyperlink ref="M94" r:id="rId93" xr:uid="{5C1389EE-7B8E-4CE1-AD67-A06B346AE661}"/>
+    <hyperlink ref="M95" r:id="rId94" xr:uid="{E6D09A0C-0E6C-4767-9502-C45CAD42E349}"/>
+    <hyperlink ref="M96" r:id="rId95" xr:uid="{3C030BC5-8750-46CD-A50B-E8D120B6AA4F}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId94"/>
+    <tablePart r:id="rId96"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 29/09/2026 13:51
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BABC0C2-4D01-402A-A898-792DA291A622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2282EF6-78F7-42D3-B924-6812D2FCE83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="471">
   <si>
     <t>ID</t>
   </si>
@@ -1423,6 +1423,18 @@
   </si>
   <si>
     <t>https://archive.org/details/1969-presentazione-il-comunista/mode/2up</t>
+  </si>
+  <si>
+    <t>AMI-0096</t>
+  </si>
+  <si>
+    <t>Pubblicità "Amaro Ramazzotti" raffigurante Mao Zedong</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/ramazzotti-1973</t>
+  </si>
+  <si>
+    <t>1973-Ramazzotti.png</t>
   </si>
 </sst>
 </file>
@@ -1848,7 +1860,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P96"/>
+  <dimension ref="A1:P97"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" customWidth="1"/>
@@ -5159,6 +5171,35 @@
       </c>
       <c r="M96" s="3" t="s">
         <v>466</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>467</v>
+      </c>
+      <c r="B97" t="s">
+        <v>468</v>
+      </c>
+      <c r="F97">
+        <v>1973</v>
+      </c>
+      <c r="G97" t="s">
+        <v>75</v>
+      </c>
+      <c r="I97" t="s">
+        <v>106</v>
+      </c>
+      <c r="J97" t="s">
+        <v>18</v>
+      </c>
+      <c r="L97" t="s">
+        <v>314</v>
+      </c>
+      <c r="M97" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="N97" t="s">
+        <v>470</v>
       </c>
     </row>
   </sheetData>
@@ -5259,10 +5300,11 @@
     <hyperlink ref="M94" r:id="rId93" xr:uid="{5C1389EE-7B8E-4CE1-AD67-A06B346AE661}"/>
     <hyperlink ref="M95" r:id="rId94" xr:uid="{E6D09A0C-0E6C-4767-9502-C45CAD42E349}"/>
     <hyperlink ref="M96" r:id="rId95" xr:uid="{3C030BC5-8750-46CD-A50B-E8D120B6AA4F}"/>
+    <hyperlink ref="M97" r:id="rId96" xr:uid="{CCEB970E-D5AA-46D9-977A-7634751F3020}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId96"/>
+    <tablePart r:id="rId97"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 02/10/2026 08:46
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2282EF6-78F7-42D3-B924-6812D2FCE83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3980230-5DB0-4446-9BE6-F7F54FEF0282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2550,7 +2550,7 @@
         <v>81</v>
       </c>
       <c r="F19" s="2">
-        <v>23511</v>
+        <v>23514</v>
       </c>
       <c r="G19" t="s">
         <v>75</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 02/10/2026 11:20
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E302D8AB-518E-4E36-99EA-1D0B0B656F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23F9D1C-20F8-49EF-97F1-AC53AA9177E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1518" uniqueCount="598">
   <si>
     <t>ID_autorita</t>
   </si>
@@ -1759,12 +1759,6 @@
     <t>gerarchica</t>
   </si>
   <si>
-    <t>attestato al 1969-10-03</t>
-  </si>
-  <si>
-    <t>Titolo di AMI-0016</t>
-  </si>
-  <si>
     <t>AMI-R-002</t>
   </si>
   <si>
@@ -1774,15 +1768,6 @@
     <t>associativa</t>
   </si>
   <si>
-    <t>attestato al 1968-08-31</t>
-  </si>
-  <si>
-    <t>Titolo di AMI-0015</t>
-  </si>
-  <si>
-    <t>Il titolo associa Pesce al partito senza indicarne la carica</t>
-  </si>
-  <si>
     <t>AMI-R-003</t>
   </si>
   <si>
@@ -1792,18 +1777,12 @@
     <t>attestato al 1968</t>
   </si>
   <si>
-    <t>Titolo di AMI-0004</t>
-  </si>
-  <si>
     <t>AMI-R-004</t>
   </si>
   <si>
     <t>organo di</t>
   </si>
   <si>
-    <t>Denominazione dell'ente</t>
-  </si>
-  <si>
     <t>AMI-R-005</t>
   </si>
   <si>
@@ -1819,17 +1798,32 @@
     <t>da definire</t>
   </si>
   <si>
-    <t>Natura del rapporto (scissione, frazione, ecc.) da documentare con una fonte</t>
-  </si>
-  <si>
     <t>Movimento</t>
+  </si>
+  <si>
+    <t>1966-1991</t>
+  </si>
+  <si>
+    <t>1966-1970</t>
+  </si>
+  <si>
+    <t>AMI-R-008</t>
+  </si>
+  <si>
+    <t>AMI-R-009</t>
+  </si>
+  <si>
+    <t>1970-1977</t>
+  </si>
+  <si>
+    <t>1977-1984</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1851,6 +1845,12 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2011,8 +2011,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4895E276-9036-4388-B350-F25B94D00A98}" name="Tabella5" displayName="Tabella5" ref="A1:J8" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:J8" xr:uid="{4895E276-9036-4388-B350-F25B94D00A98}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4895E276-9036-4388-B350-F25B94D00A98}" name="Tabella5" displayName="Tabella5" ref="A1:J10" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:J10" xr:uid="{4895E276-9036-4388-B350-F25B94D00A98}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{681E8224-5D12-4699-8FCD-F6D6D65EDFAF}" name="ID_relazione"/>
     <tableColumn id="2" xr3:uid="{ABB6B5F5-BCC1-4479-A7C9-B3517A2E96E9}" name="ID_entita_A"/>
@@ -7552,7 +7552,7 @@
         <v>396</v>
       </c>
       <c r="G26" t="s">
-        <v>599</v>
+        <v>591</v>
       </c>
       <c r="H26" t="s">
         <v>46</v>
@@ -7706,7 +7706,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
@@ -7778,15 +7778,12 @@
         <v>577</v>
       </c>
       <c r="H2" t="s">
-        <v>578</v>
-      </c>
-      <c r="I2" t="s">
-        <v>579</v>
+        <v>592</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -7801,158 +7798,187 @@
         <v>150</v>
       </c>
       <c r="F3" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="G3" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="H3" t="s">
-        <v>583</v>
-      </c>
-      <c r="I3" t="s">
-        <v>584</v>
-      </c>
-      <c r="J3" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>528</v>
+        <v>556</v>
       </c>
       <c r="E4" t="s">
-        <v>284</v>
+        <v>557</v>
       </c>
       <c r="F4" t="s">
-        <v>587</v>
+        <v>576</v>
       </c>
       <c r="G4" t="s">
         <v>577</v>
       </c>
       <c r="H4" t="s">
-        <v>588</v>
-      </c>
-      <c r="I4" t="s">
-        <v>589</v>
+        <v>596</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
       <c r="B5" t="s">
-        <v>523</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>151</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>529</v>
+        <v>549</v>
       </c>
       <c r="E5" t="s">
-        <v>150</v>
+        <v>344</v>
       </c>
       <c r="F5" t="s">
-        <v>591</v>
+        <v>576</v>
       </c>
       <c r="G5" t="s">
         <v>577</v>
       </c>
-      <c r="I5" t="s">
-        <v>592</v>
+      <c r="H5" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>593</v>
+        <v>586</v>
       </c>
       <c r="B6" t="s">
-        <v>525</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>179</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="E6" t="s">
-        <v>178</v>
+        <v>284</v>
       </c>
       <c r="F6" t="s">
-        <v>594</v>
+        <v>582</v>
       </c>
       <c r="G6" t="s">
         <v>577</v>
       </c>
-      <c r="I6" t="s">
-        <v>592</v>
+      <c r="H6" t="s">
+        <v>583</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>595</v>
+        <v>588</v>
       </c>
       <c r="B7" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="C7" t="s">
-        <v>284</v>
+        <v>151</v>
       </c>
       <c r="D7" t="s">
-        <v>536</v>
+        <v>529</v>
       </c>
       <c r="E7" t="s">
-        <v>103</v>
+        <v>150</v>
       </c>
       <c r="F7" t="s">
-        <v>591</v>
+        <v>585</v>
       </c>
       <c r="G7" t="s">
         <v>577</v>
       </c>
-      <c r="I7" t="s">
-        <v>592</v>
-      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>596</v>
+        <v>589</v>
       </c>
       <c r="B8" t="s">
+        <v>525</v>
+      </c>
+      <c r="C8" t="s">
+        <v>179</v>
+      </c>
+      <c r="D8" t="s">
+        <v>533</v>
+      </c>
+      <c r="E8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F8" t="s">
+        <v>587</v>
+      </c>
+      <c r="G8" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>594</v>
+      </c>
+      <c r="B9" t="s">
+        <v>528</v>
+      </c>
+      <c r="C9" t="s">
+        <v>284</v>
+      </c>
+      <c r="D9" t="s">
+        <v>536</v>
+      </c>
+      <c r="E9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" t="s">
+        <v>585</v>
+      </c>
+      <c r="G9" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>595</v>
+      </c>
+      <c r="B10" t="s">
         <v>539</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C10" t="s">
         <v>540</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D10" t="s">
         <v>529</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E10" t="s">
         <v>150</v>
       </c>
-      <c r="F8" t="s">
-        <v>597</v>
-      </c>
-      <c r="G8" t="s">
-        <v>597</v>
-      </c>
-      <c r="I8" t="s">
-        <v>592</v>
-      </c>
-      <c r="J8" t="s">
-        <v>598</v>
+      <c r="F10" t="s">
+        <v>590</v>
+      </c>
+      <c r="G10" t="s">
+        <v>590</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 02/10/2026 11:34
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23F9D1C-20F8-49EF-97F1-AC53AA9177E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5363FD37-321D-479C-89BE-B0C14E4CF565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1518" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1542" uniqueCount="603">
   <si>
     <t>ID_autorita</t>
   </si>
@@ -1774,9 +1774,6 @@
     <t>presidente di</t>
   </si>
   <si>
-    <t>attestato al 1968</t>
-  </si>
-  <si>
     <t>AMI-R-004</t>
   </si>
   <si>
@@ -1817,6 +1814,24 @@
   </si>
   <si>
     <t>1977-1984</t>
+  </si>
+  <si>
+    <t>1943-1976</t>
+  </si>
+  <si>
+    <t>AMI-R-010</t>
+  </si>
+  <si>
+    <t>AMI-R-011</t>
+  </si>
+  <si>
+    <t>AMI-R-012</t>
+  </si>
+  <si>
+    <t>1966-1968</t>
+  </si>
+  <si>
+    <t>1968-????</t>
   </si>
 </sst>
 </file>
@@ -2011,8 +2026,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4895E276-9036-4388-B350-F25B94D00A98}" name="Tabella5" displayName="Tabella5" ref="A1:J10" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:J10" xr:uid="{4895E276-9036-4388-B350-F25B94D00A98}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4895E276-9036-4388-B350-F25B94D00A98}" name="Tabella5" displayName="Tabella5" ref="A1:J13" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:J13" xr:uid="{4895E276-9036-4388-B350-F25B94D00A98}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{681E8224-5D12-4699-8FCD-F6D6D65EDFAF}" name="ID_relazione"/>
     <tableColumn id="2" xr3:uid="{ABB6B5F5-BCC1-4479-A7C9-B3517A2E96E9}" name="ID_entita_A"/>
@@ -7552,7 +7567,7 @@
         <v>396</v>
       </c>
       <c r="G26" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="H26" t="s">
         <v>46</v>
@@ -7706,7 +7721,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
@@ -7778,7 +7793,7 @@
         <v>577</v>
       </c>
       <c r="H2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -7804,7 +7819,7 @@
         <v>580</v>
       </c>
       <c r="H3" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -7830,12 +7845,12 @@
         <v>577</v>
       </c>
       <c r="H4" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
@@ -7856,12 +7871,12 @@
         <v>577</v>
       </c>
       <c r="H5" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
@@ -7870,10 +7885,10 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="E6" t="s">
-        <v>284</v>
+        <v>103</v>
       </c>
       <c r="F6" t="s">
         <v>582</v>
@@ -7882,87 +7897,96 @@
         <v>577</v>
       </c>
       <c r="H6" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B7" t="s">
-        <v>523</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E7" t="s">
-        <v>150</v>
+        <v>284</v>
       </c>
       <c r="F7" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="G7" t="s">
         <v>577</v>
       </c>
+      <c r="H7" t="s">
+        <v>597</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B8" t="s">
-        <v>525</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>179</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="E8" t="s">
-        <v>178</v>
+        <v>150</v>
       </c>
       <c r="F8" t="s">
-        <v>587</v>
+        <v>579</v>
       </c>
       <c r="G8" t="s">
-        <v>577</v>
+        <v>580</v>
+      </c>
+      <c r="H8" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B9" t="s">
-        <v>528</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>284</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="E9" t="s">
-        <v>103</v>
+        <v>540</v>
       </c>
       <c r="F9" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="G9" t="s">
-        <v>577</v>
+        <v>580</v>
+      </c>
+      <c r="H9" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B10" t="s">
-        <v>539</v>
+        <v>523</v>
       </c>
       <c r="C10" t="s">
-        <v>540</v>
+        <v>151</v>
       </c>
       <c r="D10" t="s">
         <v>529</v>
@@ -7971,10 +7995,79 @@
         <v>150</v>
       </c>
       <c r="F10" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
       <c r="G10" t="s">
-        <v>590</v>
+        <v>577</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>598</v>
+      </c>
+      <c r="B11" t="s">
+        <v>525</v>
+      </c>
+      <c r="C11" t="s">
+        <v>179</v>
+      </c>
+      <c r="D11" t="s">
+        <v>533</v>
+      </c>
+      <c r="E11" t="s">
+        <v>178</v>
+      </c>
+      <c r="F11" t="s">
+        <v>586</v>
+      </c>
+      <c r="G11" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>599</v>
+      </c>
+      <c r="B12" t="s">
+        <v>528</v>
+      </c>
+      <c r="C12" t="s">
+        <v>284</v>
+      </c>
+      <c r="D12" t="s">
+        <v>536</v>
+      </c>
+      <c r="E12" t="s">
+        <v>103</v>
+      </c>
+      <c r="F12" t="s">
+        <v>584</v>
+      </c>
+      <c r="G12" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>600</v>
+      </c>
+      <c r="B13" t="s">
+        <v>539</v>
+      </c>
+      <c r="C13" t="s">
+        <v>540</v>
+      </c>
+      <c r="D13" t="s">
+        <v>529</v>
+      </c>
+      <c r="E13" t="s">
+        <v>150</v>
+      </c>
+      <c r="F13" t="s">
+        <v>589</v>
+      </c>
+      <c r="G13" t="s">
+        <v>589</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 03/10/2026 11:33
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085BA701-ABC8-4E9F-89CC-9271D8166F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702E570B-72D1-497A-8918-4A2BA64DC487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2096" uniqueCount="829">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2096" uniqueCount="830">
   <si>
     <t>ID_autorita</t>
   </si>
@@ -2589,6 +2589,9 @@
   </si>
   <si>
     <t>Calcolato automaticamente dal Catalogo</t>
+  </si>
+  <si>
+    <t>Organizzazione giovanile</t>
   </si>
 </sst>
 </file>
@@ -2676,6 +2679,21 @@
   </cellStyles>
   <dxfs count="7">
     <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2705,21 +2723,6 @@
         <color auto="1"/>
         <name val="Calibri"/>
         <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
       </font>
     </dxf>
   </dxfs>
@@ -2767,13 +2770,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{59486A48-317F-495A-B99D-8ACD5E099451}" name="Tabella6" displayName="Tabella6" ref="A1:D23" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{59486A48-317F-495A-B99D-8ACD5E099451}" name="Tabella6" displayName="Tabella6" ref="A1:D23" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A1:D23" xr:uid="{59486A48-317F-495A-B99D-8ACD5E099451}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{A3615604-3D84-4F13-9671-EE093887D056}" name="Codice_ISAD" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{87E4C644-3EDF-4F45-A996-E7FF26FD6973}" name="Elemento" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{EF41A2A2-7B60-47CB-A566-55A8E2A526B2}" name="Valore" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{874121B5-A104-47D1-92CD-91A39F52BF80}" name="Note" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{A3615604-3D84-4F13-9671-EE093887D056}" name="Codice_ISAD" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{87E4C644-3EDF-4F45-A996-E7FF26FD6973}" name="Elemento" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{EF41A2A2-7B60-47CB-A566-55A8E2A526B2}" name="Valore" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{874121B5-A104-47D1-92CD-91A39F52BF80}" name="Note" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2834,7 +2837,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabella5" displayName="Tabella5" ref="A1:J13" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabella5" displayName="Tabella5" ref="A1:J13" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:J13" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="ID_relazione"/>
@@ -9349,7 +9352,7 @@
         <v>1958</v>
       </c>
       <c r="I6">
-        <v>1998</v>
+        <v>1988</v>
       </c>
       <c r="O6" t="s">
         <v>25</v>
@@ -9571,7 +9574,7 @@
         <v>57</v>
       </c>
       <c r="G12" t="s">
-        <v>53</v>
+        <v>829</v>
       </c>
       <c r="H12">
         <v>1966</v>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 03/10/2026 11:53
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702E570B-72D1-497A-8918-4A2BA64DC487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1936FDB-C378-4CD5-AA5D-73DEC29EC3DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -1085,9 +1085,6 @@
     <t>Nota del Presidente Mao sulla relazione di Kang Sheng riguardante la raccolta di materiale sulle elezioni parlamentari nei paesi capitalisti</t>
   </si>
   <si>
-    <t>Osvaldo Pesce; Mao Zedong; Dino Dini</t>
-  </si>
-  <si>
     <t>https://archive.org/details/istruzioni-mao-italiano</t>
   </si>
   <si>
@@ -2592,6 +2589,9 @@
   </si>
   <si>
     <t>Organizzazione giovanile</t>
+  </si>
+  <si>
+    <t>Osvaldo Pesce; Dino Dini</t>
   </si>
 </sst>
 </file>
@@ -4904,7 +4904,7 @@
         <v>201</v>
       </c>
       <c r="N35" t="s">
-        <v>344</v>
+        <v>829</v>
       </c>
       <c r="O35" t="s">
         <v>61</v>
@@ -4913,21 +4913,21 @@
         <v>137</v>
       </c>
       <c r="Q35" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="S35" t="s">
         <v>345</v>
       </c>
-      <c r="S35" t="s">
+      <c r="T35" t="s">
         <v>346</v>
       </c>
-      <c r="T35" t="s">
+      <c r="V35" t="s">
         <v>347</v>
-      </c>
-      <c r="V35" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B36" t="s">
         <v>139</v>
@@ -4936,7 +4936,7 @@
         <v>142</v>
       </c>
       <c r="D36" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E36" t="s">
         <v>140</v>
@@ -4945,16 +4945,16 @@
         <v>66</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J36" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="K36" t="s">
         <v>260</v>
       </c>
       <c r="L36" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M36" t="s">
         <v>201</v>
@@ -4963,15 +4963,15 @@
         <v>137</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="V36" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B37" t="s">
         <v>139</v>
@@ -4980,7 +4980,7 @@
         <v>142</v>
       </c>
       <c r="D37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E37" t="s">
         <v>140</v>
@@ -4992,19 +4992,19 @@
         <v>328</v>
       </c>
       <c r="H37" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I37" s="1">
         <v>1975</v>
       </c>
       <c r="J37" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="K37" t="s">
         <v>134</v>
       </c>
       <c r="L37" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="M37" t="s">
         <v>246</v>
@@ -5016,15 +5016,15 @@
         <v>137</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="V37" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B38" t="s">
         <v>139</v>
@@ -5033,7 +5033,7 @@
         <v>142</v>
       </c>
       <c r="D38" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E38" t="s">
         <v>140</v>
@@ -5066,15 +5066,15 @@
         <v>137</v>
       </c>
       <c r="Q38" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="V38" t="s">
         <v>365</v>
-      </c>
-      <c r="V38" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B39" t="s">
         <v>139</v>
@@ -5083,7 +5083,7 @@
         <v>142</v>
       </c>
       <c r="D39" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E39" t="s">
         <v>140</v>
@@ -5113,21 +5113,21 @@
         <v>158</v>
       </c>
       <c r="N39" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P39" t="s">
         <v>137</v>
       </c>
       <c r="Q39" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="V39" t="s">
         <v>370</v>
-      </c>
-      <c r="V39" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B40" t="s">
         <v>139</v>
@@ -5136,7 +5136,7 @@
         <v>142</v>
       </c>
       <c r="D40" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E40" t="s">
         <v>140</v>
@@ -5163,21 +5163,21 @@
         <v>135</v>
       </c>
       <c r="M40" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="P40" t="s">
         <v>137</v>
       </c>
       <c r="Q40" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="V40" t="s">
         <v>375</v>
-      </c>
-      <c r="V40" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B41" t="s">
         <v>139</v>
@@ -5186,7 +5186,7 @@
         <v>142</v>
       </c>
       <c r="D41" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E41" t="s">
         <v>140</v>
@@ -5195,7 +5195,7 @@
         <v>70</v>
       </c>
       <c r="G41" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H41" t="s">
         <v>29</v>
@@ -5219,15 +5219,15 @@
         <v>137</v>
       </c>
       <c r="Q41" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="V41" t="s">
         <v>380</v>
-      </c>
-      <c r="V41" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B42" t="s">
         <v>139</v>
@@ -5236,7 +5236,7 @@
         <v>142</v>
       </c>
       <c r="D42" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E42" t="s">
         <v>140</v>
@@ -5245,7 +5245,7 @@
         <v>133</v>
       </c>
       <c r="H42" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="I42" s="1">
         <v>1968</v>
@@ -5257,24 +5257,24 @@
         <v>134</v>
       </c>
       <c r="L42" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M42" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="P42" t="s">
         <v>137</v>
       </c>
       <c r="Q42" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="V42" t="s">
         <v>386</v>
-      </c>
-      <c r="V42" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B43" t="s">
         <v>139</v>
@@ -5283,7 +5283,7 @@
         <v>142</v>
       </c>
       <c r="D43" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E43" t="s">
         <v>140</v>
@@ -5292,7 +5292,7 @@
         <v>133</v>
       </c>
       <c r="H43" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="I43" s="1">
         <v>1967</v>
@@ -5304,13 +5304,13 @@
         <v>134</v>
       </c>
       <c r="L43" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M43" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="N43" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="O43" t="s">
         <v>22</v>
@@ -5319,15 +5319,15 @@
         <v>137</v>
       </c>
       <c r="Q43" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="V43" t="s">
         <v>392</v>
-      </c>
-      <c r="V43" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B44" t="s">
         <v>139</v>
@@ -5336,7 +5336,7 @@
         <v>142</v>
       </c>
       <c r="D44" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E44" t="s">
         <v>140</v>
@@ -5369,15 +5369,15 @@
         <v>137</v>
       </c>
       <c r="Q44" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="V44" t="s">
         <v>396</v>
-      </c>
-      <c r="V44" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B45" t="s">
         <v>139</v>
@@ -5386,7 +5386,7 @@
         <v>142</v>
       </c>
       <c r="D45" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E45" t="s">
         <v>140</v>
@@ -5419,15 +5419,15 @@
         <v>137</v>
       </c>
       <c r="Q45" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="V45" t="s">
         <v>400</v>
-      </c>
-      <c r="V45" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B46" t="s">
         <v>139</v>
@@ -5436,7 +5436,7 @@
         <v>142</v>
       </c>
       <c r="D46" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E46" t="s">
         <v>140</v>
@@ -5469,15 +5469,15 @@
         <v>137</v>
       </c>
       <c r="Q46" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="V46" t="s">
         <v>404</v>
-      </c>
-      <c r="V46" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B47" t="s">
         <v>139</v>
@@ -5486,7 +5486,7 @@
         <v>142</v>
       </c>
       <c r="D47" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E47" t="s">
         <v>140</v>
@@ -5519,15 +5519,15 @@
         <v>137</v>
       </c>
       <c r="Q47" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="V47" t="s">
         <v>408</v>
-      </c>
-      <c r="V47" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B48" t="s">
         <v>139</v>
@@ -5536,7 +5536,7 @@
         <v>142</v>
       </c>
       <c r="D48" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E48" t="s">
         <v>140</v>
@@ -5554,7 +5554,7 @@
         <v>1971</v>
       </c>
       <c r="J48" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="K48" t="s">
         <v>146</v>
@@ -5569,15 +5569,15 @@
         <v>137</v>
       </c>
       <c r="Q48" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="V48" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B49" t="s">
         <v>139</v>
@@ -5586,7 +5586,7 @@
         <v>142</v>
       </c>
       <c r="D49" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E49" t="s">
         <v>140</v>
@@ -5619,15 +5619,15 @@
         <v>137</v>
       </c>
       <c r="Q49" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="V49" t="s">
         <v>417</v>
-      </c>
-      <c r="V49" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B50" t="s">
         <v>139</v>
@@ -5636,7 +5636,7 @@
         <v>142</v>
       </c>
       <c r="D50" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E50" t="s">
         <v>140</v>
@@ -5669,15 +5669,15 @@
         <v>137</v>
       </c>
       <c r="Q50" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="V50" t="s">
         <v>421</v>
-      </c>
-      <c r="V50" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="51" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B51" t="s">
         <v>139</v>
@@ -5686,7 +5686,7 @@
         <v>142</v>
       </c>
       <c r="D51" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E51" t="s">
         <v>140</v>
@@ -5719,15 +5719,15 @@
         <v>137</v>
       </c>
       <c r="Q51" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="V51" t="s">
         <v>425</v>
-      </c>
-      <c r="V51" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B52" t="s">
         <v>139</v>
@@ -5736,7 +5736,7 @@
         <v>142</v>
       </c>
       <c r="D52" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E52" t="s">
         <v>140</v>
@@ -5769,15 +5769,15 @@
         <v>137</v>
       </c>
       <c r="Q52" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="V52" t="s">
         <v>429</v>
-      </c>
-      <c r="V52" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B53" t="s">
         <v>139</v>
@@ -5786,7 +5786,7 @@
         <v>142</v>
       </c>
       <c r="D53" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E53" t="s">
         <v>140</v>
@@ -5798,7 +5798,7 @@
         <v>80</v>
       </c>
       <c r="H53" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I53" s="1">
         <v>1969</v>
@@ -5810,7 +5810,7 @@
         <v>134</v>
       </c>
       <c r="L53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M53" t="s">
         <v>201</v>
@@ -5819,15 +5819,15 @@
         <v>137</v>
       </c>
       <c r="Q53" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="V53" t="s">
         <v>434</v>
-      </c>
-      <c r="V53" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B54" t="s">
         <v>139</v>
@@ -5836,7 +5836,7 @@
         <v>142</v>
       </c>
       <c r="D54" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E54" t="s">
         <v>140</v>
@@ -5848,13 +5848,13 @@
         <v>1972</v>
       </c>
       <c r="J54" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="K54" t="s">
         <v>231</v>
       </c>
       <c r="L54" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="M54" t="s">
         <v>201</v>
@@ -5866,15 +5866,15 @@
         <v>137</v>
       </c>
       <c r="Q54" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="V54" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B55" t="s">
         <v>139</v>
@@ -5883,7 +5883,7 @@
         <v>142</v>
       </c>
       <c r="D55" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="E55" t="s">
         <v>140</v>
@@ -5895,42 +5895,42 @@
         <v>88</v>
       </c>
       <c r="H55" t="s">
+        <v>443</v>
+      </c>
+      <c r="I55" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="I55" s="6" t="s">
+      <c r="J55" t="s">
+        <v>449</v>
+      </c>
+      <c r="K55" t="s">
         <v>445</v>
       </c>
-      <c r="J55" t="s">
-        <v>450</v>
-      </c>
-      <c r="K55" t="s">
-        <v>446</v>
-      </c>
       <c r="L55" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M55" t="s">
         <v>201</v>
       </c>
       <c r="N55" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="P55" t="s">
         <v>137</v>
       </c>
       <c r="Q55" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="R55" t="s">
         <v>448</v>
       </c>
-      <c r="R55" t="s">
-        <v>449</v>
-      </c>
       <c r="V55" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B56" t="s">
         <v>139</v>
@@ -5939,7 +5939,7 @@
         <v>142</v>
       </c>
       <c r="D56" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="E56" t="s">
         <v>140</v>
@@ -5960,7 +5960,7 @@
         <v>149</v>
       </c>
       <c r="K56" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="M56" t="s">
         <v>201</v>
@@ -5969,18 +5969,18 @@
         <v>137</v>
       </c>
       <c r="Q56" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="R56" t="s">
         <v>454</v>
       </c>
-      <c r="R56" t="s">
+      <c r="V56" t="s">
         <v>455</v>
-      </c>
-      <c r="V56" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B57" t="s">
         <v>139</v>
@@ -5989,7 +5989,7 @@
         <v>142</v>
       </c>
       <c r="D57" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E57" t="s">
         <v>140</v>
@@ -6013,24 +6013,24 @@
         <v>134</v>
       </c>
       <c r="L57" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M57" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="P57" t="s">
         <v>137</v>
       </c>
       <c r="Q57" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="V57" t="s">
         <v>459</v>
-      </c>
-      <c r="V57" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B58" t="s">
         <v>139</v>
@@ -6039,7 +6039,7 @@
         <v>142</v>
       </c>
       <c r="D58" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="E58" t="s">
         <v>212</v>
@@ -6051,45 +6051,45 @@
         <v>88</v>
       </c>
       <c r="H58" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="I58" s="2">
         <v>28253</v>
       </c>
       <c r="J58" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K58" t="s">
         <v>208</v>
       </c>
       <c r="L58" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="M58" t="s">
         <v>201</v>
       </c>
       <c r="N58" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="O58" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="P58" t="s">
         <v>137</v>
       </c>
       <c r="Q58" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="R58" t="s">
         <v>464</v>
       </c>
-      <c r="R58" t="s">
-        <v>465</v>
-      </c>
       <c r="V58" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B59" t="s">
         <v>139</v>
@@ -6098,7 +6098,7 @@
         <v>142</v>
       </c>
       <c r="D59" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="E59" t="s">
         <v>140</v>
@@ -6107,7 +6107,7 @@
         <v>32</v>
       </c>
       <c r="G59" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="H59" t="s">
         <v>32</v>
@@ -6122,7 +6122,7 @@
         <v>134</v>
       </c>
       <c r="L59" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M59" t="s">
         <v>246</v>
@@ -6131,15 +6131,15 @@
         <v>137</v>
       </c>
       <c r="Q59" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="V59" t="s">
         <v>471</v>
-      </c>
-      <c r="V59" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B60" t="s">
         <v>139</v>
@@ -6148,7 +6148,7 @@
         <v>142</v>
       </c>
       <c r="D60" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="E60" t="s">
         <v>140</v>
@@ -6157,7 +6157,7 @@
         <v>32</v>
       </c>
       <c r="G60" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="H60" t="s">
         <v>32</v>
@@ -6172,7 +6172,7 @@
         <v>134</v>
       </c>
       <c r="L60" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M60" t="s">
         <v>246</v>
@@ -6181,15 +6181,15 @@
         <v>137</v>
       </c>
       <c r="Q60" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="V60" t="s">
         <v>475</v>
-      </c>
-      <c r="V60" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B61" t="s">
         <v>139</v>
@@ -6198,7 +6198,7 @@
         <v>142</v>
       </c>
       <c r="D61" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="E61" t="s">
         <v>140</v>
@@ -6207,7 +6207,7 @@
         <v>32</v>
       </c>
       <c r="G61" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="H61" t="s">
         <v>32</v>
@@ -6216,33 +6216,33 @@
         <v>1965</v>
       </c>
       <c r="J61" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="K61" t="s">
         <v>134</v>
       </c>
       <c r="L61" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M61" t="s">
         <v>246</v>
       </c>
       <c r="N61" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="P61" t="s">
         <v>137</v>
       </c>
       <c r="Q61" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="V61" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="62" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B62" t="s">
         <v>139</v>
@@ -6251,7 +6251,7 @@
         <v>142</v>
       </c>
       <c r="D62" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="E62" t="s">
         <v>140</v>
@@ -6269,7 +6269,7 @@
         <v>1971</v>
       </c>
       <c r="J62" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="K62" t="s">
         <v>146</v>
@@ -6284,15 +6284,15 @@
         <v>137</v>
       </c>
       <c r="Q62" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="V62" t="s">
         <v>486</v>
-      </c>
-      <c r="V62" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="63" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B63" t="s">
         <v>139</v>
@@ -6301,7 +6301,7 @@
         <v>142</v>
       </c>
       <c r="D63" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="E63" t="s">
         <v>212</v>
@@ -6310,36 +6310,36 @@
         <v>24917</v>
       </c>
       <c r="J63" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="K63" t="s">
         <v>208</v>
       </c>
       <c r="L63" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="M63" t="s">
         <v>246</v>
       </c>
       <c r="O63" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="P63" t="s">
         <v>137</v>
       </c>
       <c r="Q63" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="R63" t="s">
         <v>492</v>
       </c>
-      <c r="R63" t="s">
-        <v>493</v>
-      </c>
       <c r="V63" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B64" t="s">
         <v>139</v>
@@ -6348,7 +6348,7 @@
         <v>142</v>
       </c>
       <c r="D64" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E64" t="s">
         <v>140</v>
@@ -6360,33 +6360,33 @@
         <v>83</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="J64" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="K64" t="s">
         <v>231</v>
       </c>
       <c r="L64" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="M64" t="s">
         <v>201</v>
       </c>
       <c r="P64" t="s">
+        <v>499</v>
+      </c>
+      <c r="Q64" s="3" t="s">
         <v>500</v>
       </c>
-      <c r="Q64" s="3" t="s">
-        <v>501</v>
-      </c>
       <c r="V64" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B65" t="s">
         <v>139</v>
@@ -6395,7 +6395,7 @@
         <v>142</v>
       </c>
       <c r="D65" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="E65" t="s">
         <v>140</v>
@@ -6410,30 +6410,30 @@
         <v>26956</v>
       </c>
       <c r="J65" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="K65" t="s">
         <v>231</v>
       </c>
       <c r="L65" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="M65" t="s">
         <v>201</v>
       </c>
       <c r="P65" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="Q65" s="3" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="V65" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B66" t="s">
         <v>139</v>
@@ -6442,7 +6442,7 @@
         <v>142</v>
       </c>
       <c r="D66" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="E66" t="s">
         <v>212</v>
@@ -6460,7 +6460,7 @@
         <v>208</v>
       </c>
       <c r="L66" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M66" t="s">
         <v>201</v>
@@ -6469,18 +6469,18 @@
         <v>137</v>
       </c>
       <c r="Q66" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="R66" t="s">
         <v>511</v>
       </c>
-      <c r="R66" t="s">
+      <c r="V66" t="s">
         <v>512</v>
-      </c>
-      <c r="V66" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B67" t="s">
         <v>139</v>
@@ -6489,7 +6489,7 @@
         <v>142</v>
       </c>
       <c r="D67" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="E67" t="s">
         <v>212</v>
@@ -6507,7 +6507,7 @@
         <v>208</v>
       </c>
       <c r="L67" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M67" t="s">
         <v>201</v>
@@ -6516,18 +6516,18 @@
         <v>137</v>
       </c>
       <c r="Q67" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="R67" t="s">
         <v>516</v>
       </c>
-      <c r="R67" t="s">
+      <c r="V67" t="s">
         <v>517</v>
-      </c>
-      <c r="V67" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B68" t="s">
         <v>139</v>
@@ -6536,7 +6536,7 @@
         <v>142</v>
       </c>
       <c r="D68" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="E68" t="s">
         <v>140</v>
@@ -6563,18 +6563,18 @@
         <v>137</v>
       </c>
       <c r="Q68" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="R68" t="s">
         <v>521</v>
       </c>
-      <c r="R68" t="s">
+      <c r="V68" t="s">
         <v>522</v>
-      </c>
-      <c r="V68" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B69" t="s">
         <v>139</v>
@@ -6583,7 +6583,7 @@
         <v>142</v>
       </c>
       <c r="D69" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E69" t="s">
         <v>140</v>
@@ -6595,10 +6595,10 @@
         <v>91</v>
       </c>
       <c r="I69" s="7" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="J69" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="K69" t="s">
         <v>260</v>
@@ -6613,15 +6613,15 @@
         <v>263</v>
       </c>
       <c r="Q69" s="3" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="V69" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B70" t="s">
         <v>139</v>
@@ -6630,7 +6630,7 @@
         <v>142</v>
       </c>
       <c r="D70" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E70" t="s">
         <v>140</v>
@@ -6645,7 +6645,7 @@
         <v>25704</v>
       </c>
       <c r="J70" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K70" t="s">
         <v>260</v>
@@ -6660,15 +6660,15 @@
         <v>263</v>
       </c>
       <c r="Q70" s="3" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="V70" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B71" t="s">
         <v>139</v>
@@ -6677,7 +6677,7 @@
         <v>142</v>
       </c>
       <c r="D71" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="E71" t="s">
         <v>140</v>
@@ -6692,7 +6692,7 @@
         <v>25718</v>
       </c>
       <c r="J71" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="K71" t="s">
         <v>260</v>
@@ -6707,15 +6707,15 @@
         <v>263</v>
       </c>
       <c r="Q71" s="3" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="V71" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B72" t="s">
         <v>139</v>
@@ -6724,7 +6724,7 @@
         <v>142</v>
       </c>
       <c r="D72" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E72" t="s">
         <v>140</v>
@@ -6739,7 +6739,7 @@
         <v>25719</v>
       </c>
       <c r="J72" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="K72" t="s">
         <v>260</v>
@@ -6754,15 +6754,15 @@
         <v>263</v>
       </c>
       <c r="Q72" s="3" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="V72" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B73" t="s">
         <v>139</v>
@@ -6771,7 +6771,7 @@
         <v>142</v>
       </c>
       <c r="D73" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="E73" t="s">
         <v>140</v>
@@ -6786,7 +6786,7 @@
         <v>25740</v>
       </c>
       <c r="J73" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="K73" t="s">
         <v>260</v>
@@ -6801,15 +6801,15 @@
         <v>263</v>
       </c>
       <c r="Q73" s="3" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="V73" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="74" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B74" t="s">
         <v>139</v>
@@ -6818,7 +6818,7 @@
         <v>142</v>
       </c>
       <c r="D74" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="E74" t="s">
         <v>140</v>
@@ -6833,7 +6833,7 @@
         <v>25765</v>
       </c>
       <c r="J74" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="K74" t="s">
         <v>260</v>
@@ -6848,15 +6848,15 @@
         <v>263</v>
       </c>
       <c r="Q74" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="V74" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="75" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B75" t="s">
         <v>139</v>
@@ -6865,7 +6865,7 @@
         <v>142</v>
       </c>
       <c r="D75" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="E75" t="s">
         <v>140</v>
@@ -6880,7 +6880,7 @@
         <v>25824</v>
       </c>
       <c r="J75" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="K75" t="s">
         <v>260</v>
@@ -6895,15 +6895,15 @@
         <v>263</v>
       </c>
       <c r="Q75" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="V75" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="76" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B76" t="s">
         <v>139</v>
@@ -6912,7 +6912,7 @@
         <v>142</v>
       </c>
       <c r="D76" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="E76" t="s">
         <v>140</v>
@@ -6927,7 +6927,7 @@
         <v>25866</v>
       </c>
       <c r="J76" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="K76" t="s">
         <v>260</v>
@@ -6942,15 +6942,15 @@
         <v>263</v>
       </c>
       <c r="Q76" s="3" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="V76" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="77" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B77" t="s">
         <v>139</v>
@@ -6959,7 +6959,7 @@
         <v>142</v>
       </c>
       <c r="D77" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="E77" t="s">
         <v>140</v>
@@ -6974,7 +6974,7 @@
         <v>25887</v>
       </c>
       <c r="J77" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="K77" t="s">
         <v>260</v>
@@ -6989,15 +6989,15 @@
         <v>263</v>
       </c>
       <c r="Q77" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="V77" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="78" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B78" t="s">
         <v>139</v>
@@ -7006,7 +7006,7 @@
         <v>142</v>
       </c>
       <c r="D78" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E78" t="s">
         <v>140</v>
@@ -7021,7 +7021,7 @@
         <v>25915</v>
       </c>
       <c r="J78" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="K78" t="s">
         <v>260</v>
@@ -7036,15 +7036,15 @@
         <v>263</v>
       </c>
       <c r="Q78" s="3" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="V78" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="79" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B79" t="s">
         <v>139</v>
@@ -7053,7 +7053,7 @@
         <v>142</v>
       </c>
       <c r="D79" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E79" t="s">
         <v>140</v>
@@ -7068,7 +7068,7 @@
         <v>25950</v>
       </c>
       <c r="J79" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="K79" t="s">
         <v>260</v>
@@ -7083,15 +7083,15 @@
         <v>263</v>
       </c>
       <c r="Q79" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="V79" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="80" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B80" t="s">
         <v>139</v>
@@ -7100,7 +7100,7 @@
         <v>142</v>
       </c>
       <c r="D80" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="E80" t="s">
         <v>140</v>
@@ -7115,7 +7115,7 @@
         <v>25971</v>
       </c>
       <c r="J80" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="K80" t="s">
         <v>260</v>
@@ -7130,15 +7130,15 @@
         <v>263</v>
       </c>
       <c r="Q80" s="3" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="V80" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B81" t="s">
         <v>139</v>
@@ -7147,7 +7147,7 @@
         <v>142</v>
       </c>
       <c r="D81" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E81" t="s">
         <v>140</v>
@@ -7162,7 +7162,7 @@
         <v>25999</v>
       </c>
       <c r="J81" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="K81" t="s">
         <v>260</v>
@@ -7177,15 +7177,15 @@
         <v>263</v>
       </c>
       <c r="Q81" s="3" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="V81" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B82" t="s">
         <v>139</v>
@@ -7194,7 +7194,7 @@
         <v>142</v>
       </c>
       <c r="D82" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E82" t="s">
         <v>140</v>
@@ -7209,7 +7209,7 @@
         <v>26027</v>
       </c>
       <c r="J82" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="K82" t="s">
         <v>260</v>
@@ -7224,15 +7224,15 @@
         <v>263</v>
       </c>
       <c r="Q82" s="3" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="V82" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B83" t="s">
         <v>139</v>
@@ -7241,7 +7241,7 @@
         <v>142</v>
       </c>
       <c r="D83" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="E83" t="s">
         <v>140</v>
@@ -7256,7 +7256,7 @@
         <v>26054</v>
       </c>
       <c r="J83" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="K83" t="s">
         <v>260</v>
@@ -7271,15 +7271,15 @@
         <v>263</v>
       </c>
       <c r="Q83" s="3" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="V83" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B84" t="s">
         <v>139</v>
@@ -7288,7 +7288,7 @@
         <v>142</v>
       </c>
       <c r="D84" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="E84" t="s">
         <v>140</v>
@@ -7303,7 +7303,7 @@
         <v>26076</v>
       </c>
       <c r="J84" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="K84" t="s">
         <v>260</v>
@@ -7318,15 +7318,15 @@
         <v>263</v>
       </c>
       <c r="Q84" s="3" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="V84" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B85" t="s">
         <v>139</v>
@@ -7335,7 +7335,7 @@
         <v>142</v>
       </c>
       <c r="D85" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="E85" t="s">
         <v>140</v>
@@ -7350,7 +7350,7 @@
         <v>26104</v>
       </c>
       <c r="J85" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="K85" t="s">
         <v>260</v>
@@ -7365,15 +7365,15 @@
         <v>263</v>
       </c>
       <c r="Q85" s="3" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="V85" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B86" t="s">
         <v>139</v>
@@ -7382,7 +7382,7 @@
         <v>142</v>
       </c>
       <c r="D86" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="E86" t="s">
         <v>140</v>
@@ -7397,7 +7397,7 @@
         <v>26139</v>
       </c>
       <c r="J86" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="K86" t="s">
         <v>260</v>
@@ -7412,15 +7412,15 @@
         <v>263</v>
       </c>
       <c r="Q86" s="3" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="V86" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="87" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B87" t="s">
         <v>139</v>
@@ -7429,7 +7429,7 @@
         <v>142</v>
       </c>
       <c r="D87" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E87" t="s">
         <v>140</v>
@@ -7444,7 +7444,7 @@
         <v>26265</v>
       </c>
       <c r="J87" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="K87" t="s">
         <v>260</v>
@@ -7459,15 +7459,15 @@
         <v>263</v>
       </c>
       <c r="Q87" s="3" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="V87" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="88" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B88" t="s">
         <v>139</v>
@@ -7476,7 +7476,7 @@
         <v>142</v>
       </c>
       <c r="D88" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="E88" t="s">
         <v>140</v>
@@ -7491,7 +7491,7 @@
         <v>26307</v>
       </c>
       <c r="J88" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="K88" t="s">
         <v>260</v>
@@ -7506,15 +7506,15 @@
         <v>263</v>
       </c>
       <c r="Q88" s="3" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="V88" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B89" t="s">
         <v>139</v>
@@ -7523,7 +7523,7 @@
         <v>142</v>
       </c>
       <c r="D89" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="E89" t="s">
         <v>140</v>
@@ -7538,7 +7538,7 @@
         <v>26370</v>
       </c>
       <c r="J89" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="K89" t="s">
         <v>260</v>
@@ -7553,15 +7553,15 @@
         <v>263</v>
       </c>
       <c r="Q89" s="3" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="V89" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="90" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B90" t="s">
         <v>139</v>
@@ -7570,7 +7570,7 @@
         <v>142</v>
       </c>
       <c r="D90" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="E90" t="s">
         <v>140</v>
@@ -7585,7 +7585,7 @@
         <v>26420</v>
       </c>
       <c r="J90" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="K90" t="s">
         <v>260</v>
@@ -7600,15 +7600,15 @@
         <v>263</v>
       </c>
       <c r="Q90" s="3" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="V90" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="91" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B91" t="s">
         <v>139</v>
@@ -7617,7 +7617,7 @@
         <v>142</v>
       </c>
       <c r="D91" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="E91" t="s">
         <v>140</v>
@@ -7632,7 +7632,7 @@
         <v>26608</v>
       </c>
       <c r="J91" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="K91" t="s">
         <v>260</v>
@@ -7647,15 +7647,15 @@
         <v>263</v>
       </c>
       <c r="Q91" s="3" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="V91" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="92" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B92" t="s">
         <v>139</v>
@@ -7664,7 +7664,7 @@
         <v>142</v>
       </c>
       <c r="D92" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E92" t="s">
         <v>140</v>
@@ -7679,7 +7679,7 @@
         <v>26785</v>
       </c>
       <c r="J92" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="K92" t="s">
         <v>260</v>
@@ -7694,15 +7694,15 @@
         <v>263</v>
       </c>
       <c r="Q92" s="3" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="V92" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="93" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B93" t="s">
         <v>139</v>
@@ -7711,7 +7711,7 @@
         <v>142</v>
       </c>
       <c r="D93" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="E93" t="s">
         <v>140</v>
@@ -7720,7 +7720,7 @@
         <v>66</v>
       </c>
       <c r="H93" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="I93">
         <v>1969</v>
@@ -7732,7 +7732,7 @@
         <v>134</v>
       </c>
       <c r="L93" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M93" t="s">
         <v>158</v>
@@ -7744,15 +7744,15 @@
         <v>137</v>
       </c>
       <c r="Q93" s="3" t="s">
+        <v>647</v>
+      </c>
+      <c r="V93" t="s">
         <v>648</v>
-      </c>
-      <c r="V93" t="s">
-        <v>649</v>
       </c>
     </row>
     <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B94" t="s">
         <v>139</v>
@@ -7761,7 +7761,7 @@
         <v>142</v>
       </c>
       <c r="D94" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="E94" t="s">
         <v>140</v>
@@ -7773,16 +7773,16 @@
         <v>93</v>
       </c>
       <c r="I94" s="5" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="J94" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="K94" t="s">
         <v>146</v>
       </c>
       <c r="L94" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="M94" t="s">
         <v>201</v>
@@ -7791,15 +7791,15 @@
         <v>137</v>
       </c>
       <c r="Q94" s="3" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="V94" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="95" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B95" t="s">
         <v>139</v>
@@ -7808,7 +7808,7 @@
         <v>142</v>
       </c>
       <c r="D95" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E95" t="s">
         <v>140</v>
@@ -7841,15 +7841,15 @@
         <v>159</v>
       </c>
       <c r="Q95" s="3" t="s">
+        <v>658</v>
+      </c>
+      <c r="V95" t="s">
         <v>659</v>
-      </c>
-      <c r="V95" t="s">
-        <v>660</v>
       </c>
     </row>
     <row r="96" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B96" t="s">
         <v>139</v>
@@ -7858,7 +7858,7 @@
         <v>142</v>
       </c>
       <c r="D96" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E96" t="s">
         <v>140</v>
@@ -7894,15 +7894,15 @@
         <v>159</v>
       </c>
       <c r="Q96" s="3" t="s">
+        <v>662</v>
+      </c>
+      <c r="V96" t="s">
         <v>663</v>
-      </c>
-      <c r="V96" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="97" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B97" t="s">
         <v>139</v>
@@ -7911,7 +7911,7 @@
         <v>142</v>
       </c>
       <c r="D97" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E97" t="s">
         <v>212</v>
@@ -7920,7 +7920,7 @@
         <v>1973</v>
       </c>
       <c r="J97" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="K97" t="s">
         <v>208</v>
@@ -7935,13 +7935,13 @@
         <v>137</v>
       </c>
       <c r="Q97" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="R97" t="s">
         <v>667</v>
       </c>
-      <c r="R97" t="s">
-        <v>668</v>
-      </c>
       <c r="V97" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
   </sheetData>
@@ -8063,275 +8063,275 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
+        <v>670</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>671</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>672</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>673</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
+        <v>674</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>675</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="C2" s="11" t="s">
         <v>676</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>677</v>
       </c>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>110</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="D3" s="11"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>680</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>681</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="11" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
+        <v>681</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>682</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="C5" s="11" t="s">
         <v>683</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>684</v>
       </c>
       <c r="D5" s="11"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="11" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>686</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="C7" s="11" t="s">
         <v>687</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>688</v>
       </c>
       <c r="D7" s="11"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
+        <v>688</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>689</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>690</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
+        <v>690</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>691</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>692</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="11" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
+        <v>693</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>694</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>695</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="11" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
+        <v>696</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>697</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>698</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="11" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
+        <v>699</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>700</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>701</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
+        <v>701</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>702</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="11" t="s">
         <v>703</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>704</v>
       </c>
       <c r="D13" s="11"/>
     </row>
     <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
+        <v>704</v>
+      </c>
+      <c r="B14" s="11" t="s">
         <v>705</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="C14" s="11" t="s">
         <v>706</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>707</v>
       </c>
       <c r="D14" s="11"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
+        <v>707</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>708</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="C15" s="11" t="s">
         <v>709</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>710</v>
       </c>
       <c r="D15" s="11"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
+        <v>710</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>711</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>712</v>
-      </c>
       <c r="C16" s="11" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D16" s="11"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>129</v>
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="11" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
+        <v>713</v>
+      </c>
+      <c r="B18" s="11" t="s">
         <v>714</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="C18" s="11" t="s">
         <v>715</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>716</v>
       </c>
       <c r="D18" s="11"/>
     </row>
     <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
+        <v>716</v>
+      </c>
+      <c r="B19" s="11" t="s">
         <v>717</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>718</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="11" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
+        <v>719</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>720</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="C20" s="11" t="s">
         <v>721</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>722</v>
       </c>
       <c r="D20" s="11"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
+        <v>722</v>
+      </c>
+      <c r="B21" s="11" t="s">
         <v>723</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="C21" s="11" t="s">
         <v>724</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>725</v>
       </c>
       <c r="D21" s="11"/>
     </row>
     <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
+        <v>725</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>726</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="C22" s="11" t="s">
         <v>727</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>728</v>
       </c>
       <c r="D22" s="11"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
+        <v>728</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>729</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="C23" s="11" t="s">
         <v>730</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>731</v>
       </c>
       <c r="D23" s="11"/>
     </row>
@@ -8380,22 +8380,22 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>5</v>
       </c>
       <c r="H1" t="s">
+        <v>732</v>
+      </c>
+      <c r="I1" t="s">
         <v>733</v>
-      </c>
-      <c r="I1" t="s">
-        <v>734</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="L1" s="9" t="s">
         <v>11</v>
@@ -8421,10 +8421,10 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>735</v>
+      </c>
+      <c r="B2" t="s">
         <v>736</v>
-      </c>
-      <c r="B2" t="s">
-        <v>737</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
@@ -8436,10 +8436,10 @@
         <v>133</v>
       </c>
       <c r="F2" t="s">
+        <v>737</v>
+      </c>
+      <c r="G2" t="s">
         <v>738</v>
-      </c>
-      <c r="G2" t="s">
-        <v>739</v>
       </c>
       <c r="H2">
         <v>1893</v>
@@ -8448,7 +8448,7 @@
         <v>1976</v>
       </c>
       <c r="J2" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="O2" t="s">
         <v>25</v>
@@ -8460,15 +8460,15 @@
         <v>46297</v>
       </c>
       <c r="R2" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="B3" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
@@ -8477,10 +8477,10 @@
         <v>21</v>
       </c>
       <c r="E3" t="s">
+        <v>742</v>
+      </c>
+      <c r="F3" t="s">
         <v>743</v>
-      </c>
-      <c r="F3" t="s">
-        <v>744</v>
       </c>
       <c r="H3">
         <v>1921</v>
@@ -8489,7 +8489,7 @@
         <v>1993</v>
       </c>
       <c r="J3" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="O3" t="s">
         <v>25</v>
@@ -8501,15 +8501,15 @@
         <v>46297</v>
       </c>
       <c r="R3" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B4" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
@@ -8518,10 +8518,10 @@
         <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="F4" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="H4">
         <v>1938</v>
@@ -8530,7 +8530,7 @@
         <v>2021</v>
       </c>
       <c r="J4" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="O4" t="s">
         <v>25</v>
@@ -8542,15 +8542,15 @@
         <v>46297</v>
       </c>
       <c r="R4" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B5" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -8562,7 +8562,7 @@
         <v>194</v>
       </c>
       <c r="F5" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="H5">
         <v>1931</v>
@@ -8580,15 +8580,15 @@
         <v>46297</v>
       </c>
       <c r="R5" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B6" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
@@ -8597,10 +8597,10 @@
         <v>21</v>
       </c>
       <c r="E6" t="s">
+        <v>751</v>
+      </c>
+      <c r="F6" t="s">
         <v>752</v>
-      </c>
-      <c r="F6" t="s">
-        <v>753</v>
       </c>
       <c r="H6">
         <v>1960</v>
@@ -8618,15 +8618,15 @@
         <v>46297</v>
       </c>
       <c r="R6" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B7" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
@@ -8638,7 +8638,7 @@
         <v>328</v>
       </c>
       <c r="F7" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="H7" t="s">
         <v>81</v>
@@ -8656,15 +8656,15 @@
         <v>46297</v>
       </c>
       <c r="R7" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B8" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
@@ -8673,10 +8673,10 @@
         <v>21</v>
       </c>
       <c r="E8" t="s">
+        <v>756</v>
+      </c>
+      <c r="F8" t="s">
         <v>757</v>
-      </c>
-      <c r="F8" t="s">
-        <v>758</v>
       </c>
       <c r="H8" t="s">
         <v>81</v>
@@ -8694,15 +8694,15 @@
         <v>46297</v>
       </c>
       <c r="R8" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="B9" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
@@ -8711,13 +8711,13 @@
         <v>21</v>
       </c>
       <c r="E9" t="s">
+        <v>759</v>
+      </c>
+      <c r="F9" t="s">
         <v>760</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>761</v>
-      </c>
-      <c r="G9" t="s">
-        <v>762</v>
       </c>
       <c r="H9">
         <v>1907</v>
@@ -8735,15 +8735,15 @@
         <v>46297</v>
       </c>
       <c r="R9" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B10" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
@@ -8752,10 +8752,10 @@
         <v>21</v>
       </c>
       <c r="E10" t="s">
+        <v>763</v>
+      </c>
+      <c r="F10" t="s">
         <v>764</v>
-      </c>
-      <c r="F10" t="s">
-        <v>765</v>
       </c>
       <c r="H10">
         <v>1898</v>
@@ -8773,15 +8773,15 @@
         <v>46297</v>
       </c>
       <c r="R10" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="B11" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C11" t="s">
         <v>20</v>
@@ -8790,13 +8790,13 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
+        <v>766</v>
+      </c>
+      <c r="F11" t="s">
         <v>767</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>768</v>
-      </c>
-      <c r="G11" t="s">
-        <v>769</v>
       </c>
       <c r="H11">
         <v>1898</v>
@@ -8814,15 +8814,15 @@
         <v>46297</v>
       </c>
       <c r="R11" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="B12" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C12" t="s">
         <v>20</v>
@@ -8831,13 +8831,13 @@
         <v>21</v>
       </c>
       <c r="E12" t="s">
+        <v>770</v>
+      </c>
+      <c r="F12" t="s">
         <v>771</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>772</v>
-      </c>
-      <c r="G12" t="s">
-        <v>773</v>
       </c>
       <c r="H12">
         <v>1904</v>
@@ -8855,15 +8855,15 @@
         <v>46297</v>
       </c>
       <c r="R12" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B13" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
@@ -8872,13 +8872,13 @@
         <v>21</v>
       </c>
       <c r="E13" t="s">
+        <v>774</v>
+      </c>
+      <c r="F13" t="s">
         <v>775</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>776</v>
-      </c>
-      <c r="G13" t="s">
-        <v>777</v>
       </c>
       <c r="H13">
         <v>1914</v>
@@ -8896,15 +8896,15 @@
         <v>46297</v>
       </c>
       <c r="R13" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B14" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
@@ -8913,10 +8913,10 @@
         <v>21</v>
       </c>
       <c r="E14" t="s">
+        <v>778</v>
+      </c>
+      <c r="F14" t="s">
         <v>779</v>
-      </c>
-      <c r="F14" t="s">
-        <v>780</v>
       </c>
       <c r="H14">
         <v>1920</v>
@@ -8934,15 +8934,15 @@
         <v>46297</v>
       </c>
       <c r="R14" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B15" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
@@ -8951,10 +8951,10 @@
         <v>21</v>
       </c>
       <c r="E15" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="F15" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="H15">
         <v>1920</v>
@@ -8972,15 +8972,15 @@
         <v>46297</v>
       </c>
       <c r="R15" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="B16" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C16" t="s">
         <v>20</v>
@@ -8989,13 +8989,13 @@
         <v>21</v>
       </c>
       <c r="E16" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F16" t="s">
+        <v>783</v>
+      </c>
+      <c r="G16" t="s">
         <v>784</v>
-      </c>
-      <c r="G16" t="s">
-        <v>785</v>
       </c>
       <c r="H16">
         <v>1898</v>
@@ -9013,15 +9013,15 @@
         <v>46297</v>
       </c>
       <c r="R16" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="B17" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
@@ -9030,10 +9030,10 @@
         <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F17" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="H17">
         <v>1924</v>
@@ -9051,15 +9051,15 @@
         <v>46297</v>
       </c>
       <c r="R17" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B18" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C18" t="s">
         <v>20</v>
@@ -9068,10 +9068,10 @@
         <v>21</v>
       </c>
       <c r="E18" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F18" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="H18">
         <v>1933</v>
@@ -9089,7 +9089,7 @@
         <v>46297</v>
       </c>
       <c r="R18" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
   </sheetData>
@@ -9574,7 +9574,7 @@
         <v>57</v>
       </c>
       <c r="G12" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="H12">
         <v>1966</v>
@@ -10306,45 +10306,45 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
+        <v>789</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>790</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="9" t="s">
         <v>791</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>792</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>793</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>794</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>795</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
+        <v>680</v>
+      </c>
+      <c r="I1" s="9" t="s">
         <v>796</v>
       </c>
-      <c r="H1" s="9" t="s">
-        <v>681</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>797</v>
-      </c>
       <c r="J1" s="9" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B2" t="s">
+        <v>741</v>
+      </c>
+      <c r="C2" t="s">
         <v>742</v>
-      </c>
-      <c r="C2" t="s">
-        <v>743</v>
       </c>
       <c r="D2" t="s">
         <v>60</v>
@@ -10353,24 +10353,24 @@
         <v>61</v>
       </c>
       <c r="F2" t="s">
+        <v>798</v>
+      </c>
+      <c r="G2" t="s">
         <v>799</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>800</v>
-      </c>
-      <c r="H2" t="s">
-        <v>801</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="B3" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="C3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D3" t="s">
         <v>60</v>
@@ -10379,24 +10379,24 @@
         <v>61</v>
       </c>
       <c r="F3" t="s">
+        <v>802</v>
+      </c>
+      <c r="G3" t="s">
         <v>803</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>804</v>
-      </c>
-      <c r="H3" t="s">
-        <v>805</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B4" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="C4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D4" t="s">
         <v>100</v>
@@ -10405,24 +10405,24 @@
         <v>101</v>
       </c>
       <c r="F4" t="s">
+        <v>798</v>
+      </c>
+      <c r="G4" t="s">
         <v>799</v>
       </c>
-      <c r="G4" t="s">
-        <v>800</v>
-      </c>
       <c r="H4" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B5" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="C5" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D5" t="s">
         <v>87</v>
@@ -10431,21 +10431,21 @@
         <v>88</v>
       </c>
       <c r="F5" t="s">
+        <v>798</v>
+      </c>
+      <c r="G5" t="s">
         <v>799</v>
       </c>
-      <c r="G5" t="s">
-        <v>800</v>
-      </c>
       <c r="H5" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B6" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C6" t="s">
         <v>133</v>
@@ -10457,21 +10457,21 @@
         <v>70</v>
       </c>
       <c r="F6" t="s">
+        <v>810</v>
+      </c>
+      <c r="G6" t="s">
+        <v>799</v>
+      </c>
+      <c r="H6" t="s">
         <v>811</v>
-      </c>
-      <c r="G6" t="s">
-        <v>800</v>
-      </c>
-      <c r="H6" t="s">
-        <v>812</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B7" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C7" t="s">
         <v>133</v>
@@ -10483,24 +10483,24 @@
         <v>59</v>
       </c>
       <c r="F7" t="s">
+        <v>810</v>
+      </c>
+      <c r="G7" t="s">
+        <v>799</v>
+      </c>
+      <c r="H7" t="s">
         <v>811</v>
-      </c>
-      <c r="G7" t="s">
-        <v>800</v>
-      </c>
-      <c r="H7" t="s">
-        <v>812</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B8" t="s">
+        <v>755</v>
+      </c>
+      <c r="C8" t="s">
         <v>756</v>
-      </c>
-      <c r="C8" t="s">
-        <v>757</v>
       </c>
       <c r="D8" t="s">
         <v>60</v>
@@ -10509,24 +10509,24 @@
         <v>61</v>
       </c>
       <c r="F8" t="s">
+        <v>802</v>
+      </c>
+      <c r="G8" t="s">
         <v>803</v>
       </c>
-      <c r="G8" t="s">
-        <v>804</v>
-      </c>
       <c r="H8" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="B9" t="s">
+        <v>755</v>
+      </c>
+      <c r="C9" t="s">
         <v>756</v>
-      </c>
-      <c r="C9" t="s">
-        <v>757</v>
       </c>
       <c r="D9" t="s">
         <v>73</v>
@@ -10535,18 +10535,18 @@
         <v>74</v>
       </c>
       <c r="F9" t="s">
+        <v>802</v>
+      </c>
+      <c r="G9" t="s">
         <v>803</v>
       </c>
-      <c r="G9" t="s">
-        <v>804</v>
-      </c>
       <c r="H9" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B10" t="s">
         <v>51</v>
@@ -10561,15 +10561,15 @@
         <v>61</v>
       </c>
       <c r="F10" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="G10" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B11" t="s">
         <v>54</v>
@@ -10584,15 +10584,15 @@
         <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="G11" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B12" t="s">
         <v>58</v>
@@ -10607,15 +10607,15 @@
         <v>70</v>
       </c>
       <c r="F12" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="G12" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B13" t="s">
         <v>73</v>
@@ -10630,10 +10630,10 @@
         <v>61</v>
       </c>
       <c r="F13" t="s">
+        <v>823</v>
+      </c>
+      <c r="G13" t="s">
         <v>824</v>
-      </c>
-      <c r="G13" t="s">
-        <v>825</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 04/10/2026 11:31
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{041153CE-BB4E-499A-8E40-EBA3A27C5714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCCB5099-04C0-43FF-8CAA-FD03A5D0D9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2753" uniqueCount="1069">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2684" uniqueCount="1050">
   <si>
     <t>ID_autorita</t>
   </si>
@@ -2799,9 +2799,6 @@
     <t>Coscienza Operaia</t>
   </si>
   <si>
-    <t>AMI-O-031</t>
-  </si>
-  <si>
     <t>Federazione Marxista-Leninista d'Italia</t>
   </si>
   <si>
@@ -2868,9 +2865,6 @@
     <t>Categoria_ISAAR</t>
   </si>
   <si>
-    <t>Fonte</t>
-  </si>
-  <si>
     <t>AMI-R-001</t>
   </si>
   <si>
@@ -2883,9 +2877,6 @@
     <t>1966-1991</t>
   </si>
   <si>
-    <t>AMI-0013; AMI-0016</t>
-  </si>
-  <si>
     <t>AMI-R-002</t>
   </si>
   <si>
@@ -2898,9 +2889,6 @@
     <t>1966-1970</t>
   </si>
   <si>
-    <t>AMI-0014; AMI-0033</t>
-  </si>
-  <si>
     <t>AMI-R-003</t>
   </si>
   <si>
@@ -2913,9 +2901,6 @@
     <t>1977-1984</t>
   </si>
   <si>
-    <t>AMI-0057; AMI-0054</t>
-  </si>
-  <si>
     <t>AMI-R-005</t>
   </si>
   <si>
@@ -2967,9 +2952,6 @@
     <t>AMI-R-013</t>
   </si>
   <si>
-    <t>AMI-0032; AMI-0036</t>
-  </si>
-  <si>
     <t>AMI-R-014</t>
   </si>
   <si>
@@ -2979,18 +2961,9 @@
     <t>temporale</t>
   </si>
   <si>
-    <t>1976</t>
-  </si>
-  <si>
     <t>AMI-R-015</t>
   </si>
   <si>
-    <t>prima del 1969</t>
-  </si>
-  <si>
-    <t>Tipo di entità da verificare (gruppo o testata)</t>
-  </si>
-  <si>
     <t>AMI-R-016</t>
   </si>
   <si>
@@ -3000,9 +2973,6 @@
     <t>AMI-R-018</t>
   </si>
   <si>
-    <t>attestato 1967</t>
-  </si>
-  <si>
     <t>AMI-R-019</t>
   </si>
   <si>
@@ -3012,60 +2982,24 @@
     <t>AMI-R-020</t>
   </si>
   <si>
-    <t>rappresentante di</t>
-  </si>
-  <si>
-    <t>1964</t>
-  </si>
-  <si>
-    <t>Nome di battaglia "Livio": da registrare come variante</t>
-  </si>
-  <si>
     <t>AMI-R-021</t>
   </si>
   <si>
-    <t>Variante del nome: "Gino"</t>
-  </si>
-  <si>
     <t>AMI-R-022</t>
   </si>
   <si>
-    <t>casa editrice di</t>
-  </si>
-  <si>
-    <t>attestato 1969</t>
-  </si>
-  <si>
-    <t>AMI-0035; AMI-0092</t>
-  </si>
-  <si>
-    <t>AMI-R-023</t>
-  </si>
-  <si>
-    <t>AMI-0053; AMI-0063</t>
-  </si>
-  <si>
     <t>AMI-R-024</t>
   </si>
   <si>
-    <t>La fonte dice "UCI di Aldo Brandirali"</t>
-  </si>
-  <si>
     <t>AMI-R-025</t>
   </si>
   <si>
-    <t>attestato 1974</t>
-  </si>
-  <si>
     <t>AMI-R-026</t>
   </si>
   <si>
     <t>dirigente di</t>
   </si>
   <si>
-    <t>La fonte dice "animato da"</t>
-  </si>
-  <si>
     <t>AMI-R-027</t>
   </si>
   <si>
@@ -3111,12 +3045,6 @@
     <t>AMI-R-037</t>
   </si>
   <si>
-    <t>AMI-0057; AMI-0064</t>
-  </si>
-  <si>
-    <t>Variante del nome: "Beppe"</t>
-  </si>
-  <si>
     <t>AMI-R-038</t>
   </si>
   <si>
@@ -3126,78 +3054,42 @@
     <t>organo di stampa di</t>
   </si>
   <si>
-    <t>dal 1977</t>
-  </si>
-  <si>
     <t>AMI-R-040</t>
   </si>
   <si>
-    <t>fino al 1977</t>
-  </si>
-  <si>
     <t>AMI-R-041</t>
   </si>
   <si>
-    <t>Anno 1973 ricavato da AMI-0057 ("nata nel 1973")</t>
-  </si>
-  <si>
     <t>AMI-R-042</t>
   </si>
   <si>
-    <t>Testata omonima dell'organizzazione</t>
-  </si>
-  <si>
     <t>AMI-R-043</t>
   </si>
   <si>
-    <t>attestato 1970</t>
-  </si>
-  <si>
     <t>AMI-R-044</t>
   </si>
   <si>
     <t>curatore di</t>
   </si>
   <si>
-    <t>come sopra</t>
-  </si>
-  <si>
     <t>AMI-R-045</t>
   </si>
   <si>
     <t>derivato da</t>
   </si>
   <si>
-    <t>La descrizione cita come fonte BFS collezioni digitali (fonte secondaria)</t>
-  </si>
-  <si>
     <t>AMI-R-046</t>
   </si>
   <si>
-    <t>Con i Circoli Lenin toscani; fonte BFS come sopra</t>
-  </si>
-  <si>
     <t>AMI-R-047</t>
   </si>
   <si>
-    <t>attestato 1965</t>
-  </si>
-  <si>
     <t>AMI-R-048</t>
   </si>
   <si>
-    <t>attestato 1968</t>
-  </si>
-  <si>
     <t>AMI-R-049</t>
   </si>
   <si>
-    <t>1966</t>
-  </si>
-  <si>
-    <t>Infografica AMI «Il marxismo-leninismo italiano»</t>
-  </si>
-  <si>
     <t>AMI-R-050</t>
   </si>
   <si>
@@ -3291,9 +3183,6 @@
     <t>Il Partito</t>
   </si>
   <si>
-    <t>-1973</t>
-  </si>
-  <si>
     <t>AMI-R-067</t>
   </si>
   <si>
@@ -3307,13 +3196,67 @@
   </si>
   <si>
     <t>giovanile di</t>
+  </si>
+  <si>
+    <t>UGCd'I(m-l)</t>
+  </si>
+  <si>
+    <t>Dino Frangioni; Giacomo Monemezzani</t>
+  </si>
+  <si>
+    <t>1921-</t>
+  </si>
+  <si>
+    <t>1966-1967</t>
+  </si>
+  <si>
+    <t>1968-1969</t>
+  </si>
+  <si>
+    <t>1969-1976</t>
+  </si>
+  <si>
+    <t>1976-1981</t>
+  </si>
+  <si>
+    <t>1962-1963</t>
+  </si>
+  <si>
+    <t>AMI-R-069</t>
+  </si>
+  <si>
+    <t>1962-2010</t>
+  </si>
+  <si>
+    <t>1964-1966</t>
+  </si>
+  <si>
+    <t>1968-1972</t>
+  </si>
+  <si>
+    <t>1969-1977</t>
+  </si>
+  <si>
+    <t>1968-1977</t>
+  </si>
+  <si>
+    <t>1969-1973</t>
+  </si>
+  <si>
+    <t>1970-1973</t>
+  </si>
+  <si>
+    <t>1968-1976</t>
+  </si>
+  <si>
+    <t>1973-1977</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3341,6 +3284,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Georgia"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -3373,7 +3322,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -3387,6 +3336,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -3549,9 +3499,9 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabella5" displayName="Tabella5" ref="A1:J84" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:J84" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabella5" displayName="Tabella5" ref="A1:H84" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:H84" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="ID_relazione"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="ID_entita_A"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Entita_A"/>
@@ -3560,8 +3510,6 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Relazione"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Categoria_ISAAR"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Date"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Fonte"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4854,6 +4802,9 @@
       <c r="M19" t="s">
         <v>233</v>
       </c>
+      <c r="N19" s="11" t="s">
+        <v>1033</v>
+      </c>
       <c r="P19" t="s">
         <v>172</v>
       </c>
@@ -5376,6 +5327,9 @@
       </c>
       <c r="M30" t="s">
         <v>304</v>
+      </c>
+      <c r="N30" t="s">
+        <v>86</v>
       </c>
       <c r="O30" t="s">
         <v>354</v>
@@ -8870,8 +8824,9 @@
     <hyperlink ref="Q97" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId97"/>
   <tableParts count="1">
-    <tablePart r:id="rId97"/>
+    <tablePart r:id="rId98"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10788,6 +10743,9 @@
       <c r="E12" t="s">
         <v>845</v>
       </c>
+      <c r="F12" t="s">
+        <v>1032</v>
+      </c>
       <c r="G12" t="s">
         <v>846</v>
       </c>
@@ -11573,7 +11531,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
@@ -11589,41 +11547,35 @@
     <col min="12" max="12" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
+        <v>914</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>915</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="9" t="s">
         <v>916</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>917</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>918</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>919</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>920</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>921</v>
       </c>
       <c r="H1" s="9" t="s">
         <v>754</v>
       </c>
-      <c r="I1" s="9" t="s">
-        <v>922</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>747</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="B2" t="s">
         <v>31</v>
@@ -11638,21 +11590,18 @@
         <v>229</v>
       </c>
       <c r="F2" t="s">
+        <v>922</v>
+      </c>
+      <c r="G2" t="s">
+        <v>923</v>
+      </c>
+      <c r="H2" t="s">
         <v>924</v>
       </c>
-      <c r="G2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>925</v>
-      </c>
-      <c r="H2" t="s">
-        <v>926</v>
-      </c>
-      <c r="I2" t="s">
-        <v>927</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>928</v>
       </c>
       <c r="B3" t="s">
         <v>36</v>
@@ -11667,21 +11616,18 @@
         <v>229</v>
       </c>
       <c r="F3" t="s">
+        <v>926</v>
+      </c>
+      <c r="G3" t="s">
+        <v>927</v>
+      </c>
+      <c r="H3" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>929</v>
-      </c>
-      <c r="G3" t="s">
-        <v>930</v>
-      </c>
-      <c r="H3" t="s">
-        <v>931</v>
-      </c>
-      <c r="I3" t="s">
-        <v>932</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>933</v>
       </c>
       <c r="B4" t="s">
         <v>36</v>
@@ -11696,21 +11642,18 @@
         <v>887</v>
       </c>
       <c r="F4" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="G4" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H4" t="s">
-        <v>934</v>
-      </c>
-      <c r="I4" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>935</v>
+        <v>931</v>
       </c>
       <c r="B5" t="s">
         <v>36</v>
@@ -11725,21 +11668,18 @@
         <v>505</v>
       </c>
       <c r="F5" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="G5" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H5" t="s">
-        <v>936</v>
-      </c>
-      <c r="I5" t="s">
-        <v>937</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
@@ -11754,21 +11694,18 @@
         <v>166</v>
       </c>
       <c r="F6" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="G6" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H6" t="s">
-        <v>940</v>
-      </c>
-      <c r="I6" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
       <c r="B7" t="s">
         <v>18</v>
@@ -11783,21 +11720,18 @@
         <v>412</v>
       </c>
       <c r="F7" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="G7" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H7" t="s">
-        <v>940</v>
-      </c>
-      <c r="I7" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="B8" t="s">
         <v>53</v>
@@ -11812,21 +11746,18 @@
         <v>229</v>
       </c>
       <c r="F8" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G8" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H8" t="s">
-        <v>943</v>
-      </c>
-      <c r="I8" t="s">
-        <v>932</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
       <c r="B9" t="s">
         <v>53</v>
@@ -11841,18 +11772,18 @@
         <v>867</v>
       </c>
       <c r="F9" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G9" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H9" t="s">
-        <v>945</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="B10" t="s">
         <v>841</v>
@@ -11867,15 +11798,18 @@
         <v>229</v>
       </c>
       <c r="F10" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="G10" t="s">
-        <v>925</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+      <c r="H10" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>948</v>
+        <v>943</v>
       </c>
       <c r="B11" t="s">
         <v>843</v>
@@ -11890,15 +11824,15 @@
         <v>267</v>
       </c>
       <c r="F11" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
       <c r="G11" t="s">
-        <v>925</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
       <c r="B12" t="s">
         <v>847</v>
@@ -11913,15 +11847,18 @@
         <v>166</v>
       </c>
       <c r="F12" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="G12" t="s">
-        <v>925</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+      <c r="H12" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
       <c r="B13" t="s">
         <v>866</v>
@@ -11936,15 +11873,18 @@
         <v>229</v>
       </c>
       <c r="F13" t="s">
-        <v>952</v>
+        <v>947</v>
       </c>
       <c r="G13" t="s">
-        <v>953</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>948</v>
+      </c>
+      <c r="H13">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>954</v>
+        <v>949</v>
       </c>
       <c r="B14" t="s">
         <v>49</v>
@@ -11959,21 +11899,18 @@
         <v>369</v>
       </c>
       <c r="F14" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="G14" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H14" t="s">
-        <v>168</v>
-      </c>
-      <c r="I14" t="s">
-        <v>955</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>956</v>
+        <v>950</v>
       </c>
       <c r="B15" t="s">
         <v>869</v>
@@ -11982,24 +11919,21 @@
         <v>369</v>
       </c>
       <c r="E15" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="F15" t="s">
-        <v>957</v>
+        <v>951</v>
       </c>
       <c r="G15" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H15" t="s">
-        <v>959</v>
-      </c>
-      <c r="I15" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>960</v>
+        <v>953</v>
       </c>
       <c r="B16" t="s">
         <v>49</v>
@@ -12008,27 +11942,21 @@
         <v>50</v>
       </c>
       <c r="E16" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F16" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G16" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H16" t="s">
-        <v>961</v>
-      </c>
-      <c r="I16" t="s">
-        <v>367</v>
-      </c>
-      <c r="J16" t="s">
-        <v>962</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>963</v>
+        <v>954</v>
       </c>
       <c r="B17" t="s">
         <v>49</v>
@@ -12037,24 +11965,21 @@
         <v>50</v>
       </c>
       <c r="E17" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="F17" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G17" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H17" t="s">
-        <v>961</v>
-      </c>
-      <c r="I17" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>964</v>
+        <v>955</v>
       </c>
       <c r="B18" t="s">
         <v>49</v>
@@ -12063,27 +11988,21 @@
         <v>50</v>
       </c>
       <c r="E18" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F18" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G18" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H18" t="s">
-        <v>961</v>
-      </c>
-      <c r="I18" t="s">
-        <v>367</v>
-      </c>
-      <c r="J18" t="s">
-        <v>962</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>965</v>
+        <v>956</v>
       </c>
       <c r="B19" t="s">
         <v>90</v>
@@ -12098,21 +12017,18 @@
         <v>439</v>
       </c>
       <c r="F19" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="G19" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H19" t="s">
-        <v>966</v>
-      </c>
-      <c r="I19" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>967</v>
+        <v>957</v>
       </c>
       <c r="B20" t="s">
         <v>90</v>
@@ -12121,24 +12037,21 @@
         <v>91</v>
       </c>
       <c r="E20" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F20" t="s">
-        <v>968</v>
+        <v>958</v>
       </c>
       <c r="G20" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H20" t="s">
-        <v>966</v>
-      </c>
-      <c r="I20" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>969</v>
+        <v>959</v>
       </c>
       <c r="B21" t="s">
         <v>115</v>
@@ -12147,88 +12060,73 @@
         <v>116</v>
       </c>
       <c r="D21" t="s">
+        <v>850</v>
+      </c>
+      <c r="E21" t="s">
+        <v>229</v>
+      </c>
+      <c r="F21" t="s">
+        <v>926</v>
+      </c>
+      <c r="G21" t="s">
+        <v>927</v>
+      </c>
+      <c r="H21">
+        <v>1966</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>960</v>
+      </c>
+      <c r="B22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" t="s">
         <v>821</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E22" t="s">
         <v>276</v>
       </c>
-      <c r="F21" t="s">
-        <v>970</v>
-      </c>
-      <c r="G21" t="s">
-        <v>930</v>
-      </c>
-      <c r="H21" t="s">
-        <v>971</v>
-      </c>
-      <c r="I21" t="s">
-        <v>274</v>
-      </c>
-      <c r="J21" t="s">
-        <v>972</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>973</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="F22" t="s">
+        <v>926</v>
+      </c>
+      <c r="G22" t="s">
+        <v>927</v>
+      </c>
+      <c r="H22" t="s">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>961</v>
+      </c>
+      <c r="B23" t="s">
         <v>119</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C23" t="s">
         <v>120</v>
       </c>
-      <c r="E22" t="s">
-        <v>903</v>
-      </c>
-      <c r="F22" t="s">
-        <v>970</v>
-      </c>
-      <c r="G22" t="s">
-        <v>930</v>
-      </c>
-      <c r="H22" t="s">
-        <v>971</v>
-      </c>
-      <c r="I22" t="s">
-        <v>274</v>
-      </c>
-      <c r="J22" t="s">
-        <v>974</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>975</v>
-      </c>
-      <c r="B23" t="s">
-        <v>899</v>
-      </c>
-      <c r="C23" t="s">
-        <v>715</v>
-      </c>
-      <c r="D23" t="s">
-        <v>856</v>
-      </c>
       <c r="E23" t="s">
-        <v>267</v>
+        <v>902</v>
       </c>
       <c r="F23" t="s">
-        <v>976</v>
+        <v>926</v>
       </c>
       <c r="G23" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H23" t="s">
-        <v>977</v>
-      </c>
-      <c r="I23" t="s">
-        <v>978</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>979</v>
+        <v>962</v>
       </c>
       <c r="B24" t="s">
         <v>856</v>
@@ -12243,21 +12141,18 @@
         <v>500</v>
       </c>
       <c r="F24" t="s">
-        <v>957</v>
+        <v>951</v>
       </c>
       <c r="G24" t="s">
-        <v>958</v>
-      </c>
-      <c r="H24" t="s">
-        <v>498</v>
-      </c>
-      <c r="I24" t="s">
-        <v>980</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+        <v>952</v>
+      </c>
+      <c r="H24">
+        <v>1972</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="B25" t="s">
         <v>109</v>
@@ -12272,21 +12167,18 @@
         <v>267</v>
       </c>
       <c r="F25" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="G25" t="s">
-        <v>925</v>
-      </c>
-      <c r="I25" t="s">
-        <v>560</v>
-      </c>
-      <c r="J25" t="s">
-        <v>982</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+      <c r="H25" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>983</v>
+        <v>964</v>
       </c>
       <c r="B26" t="s">
         <v>895</v>
@@ -12301,21 +12193,15 @@
         <v>500</v>
       </c>
       <c r="F26" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
       <c r="G26" t="s">
-        <v>925</v>
-      </c>
-      <c r="H26" t="s">
-        <v>984</v>
-      </c>
-      <c r="I26" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>985</v>
+        <v>966</v>
       </c>
       <c r="B27" t="s">
         <v>123</v>
@@ -12330,21 +12216,18 @@
         <v>491</v>
       </c>
       <c r="F27" t="s">
-        <v>986</v>
+        <v>965</v>
       </c>
       <c r="G27" t="s">
-        <v>925</v>
-      </c>
-      <c r="I27" t="s">
-        <v>489</v>
-      </c>
-      <c r="J27" t="s">
-        <v>987</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+      <c r="H27" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>988</v>
+        <v>967</v>
       </c>
       <c r="B28" t="s">
         <v>136</v>
@@ -12359,18 +12242,18 @@
         <v>491</v>
       </c>
       <c r="F28" t="s">
-        <v>986</v>
+        <v>965</v>
       </c>
       <c r="G28" t="s">
-        <v>925</v>
-      </c>
-      <c r="I28" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+      <c r="H28" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>989</v>
+        <v>969</v>
       </c>
       <c r="B29" t="s">
         <v>871</v>
@@ -12379,24 +12262,21 @@
         <v>491</v>
       </c>
       <c r="E29" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="F29" t="s">
-        <v>990</v>
+        <v>968</v>
       </c>
       <c r="G29" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H29" t="s">
         <v>184</v>
       </c>
-      <c r="I29" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>991</v>
+        <v>970</v>
       </c>
       <c r="B30" t="s">
         <v>892</v>
@@ -12411,21 +12291,18 @@
         <v>491</v>
       </c>
       <c r="F30" t="s">
+        <v>947</v>
+      </c>
+      <c r="G30" t="s">
         <v>952</v>
-      </c>
-      <c r="G30" t="s">
-        <v>958</v>
       </c>
       <c r="H30" t="s">
         <v>168</v>
       </c>
-      <c r="I30" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>992</v>
+        <v>971</v>
       </c>
       <c r="B31" t="s">
         <v>136</v>
@@ -12440,18 +12317,18 @@
         <v>893</v>
       </c>
       <c r="F31" t="s">
-        <v>986</v>
+        <v>965</v>
       </c>
       <c r="G31" t="s">
-        <v>925</v>
-      </c>
-      <c r="I31" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+      <c r="H31" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>993</v>
+        <v>974</v>
       </c>
       <c r="B32" t="s">
         <v>886</v>
@@ -12466,21 +12343,18 @@
         <v>505</v>
       </c>
       <c r="F32" t="s">
-        <v>994</v>
+        <v>972</v>
       </c>
       <c r="G32" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H32" t="s">
-        <v>995</v>
-      </c>
-      <c r="I32" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>996</v>
+        <v>975</v>
       </c>
       <c r="B33" t="s">
         <v>880</v>
@@ -12495,21 +12369,18 @@
         <v>505</v>
       </c>
       <c r="F33" t="s">
-        <v>994</v>
+        <v>972</v>
       </c>
       <c r="G33" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H33" t="s">
-        <v>995</v>
-      </c>
-      <c r="I33" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>997</v>
+        <v>977</v>
       </c>
       <c r="B34" t="s">
         <v>889</v>
@@ -12524,21 +12395,18 @@
         <v>505</v>
       </c>
       <c r="F34" t="s">
-        <v>998</v>
+        <v>976</v>
       </c>
       <c r="G34" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H34" t="s">
-        <v>995</v>
-      </c>
-      <c r="I34" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>999</v>
+        <v>978</v>
       </c>
       <c r="B35" t="s">
         <v>892</v>
@@ -12553,21 +12421,18 @@
         <v>505</v>
       </c>
       <c r="F35" t="s">
-        <v>998</v>
+        <v>976</v>
       </c>
       <c r="G35" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H35" t="s">
-        <v>995</v>
-      </c>
-      <c r="I35" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1000</v>
+        <v>979</v>
       </c>
       <c r="B36" t="s">
         <v>897</v>
@@ -12582,27 +12447,24 @@
         <v>505</v>
       </c>
       <c r="F36" t="s">
-        <v>998</v>
+        <v>976</v>
       </c>
       <c r="G36" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H36" t="s">
-        <v>995</v>
-      </c>
-      <c r="I36" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1001</v>
+        <v>980</v>
       </c>
       <c r="B37" t="s">
+        <v>903</v>
+      </c>
+      <c r="C37" t="s">
         <v>904</v>
-      </c>
-      <c r="C37" t="s">
-        <v>905</v>
       </c>
       <c r="D37" t="s">
         <v>875</v>
@@ -12611,21 +12473,18 @@
         <v>505</v>
       </c>
       <c r="F37" t="s">
-        <v>998</v>
+        <v>976</v>
       </c>
       <c r="G37" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H37" t="s">
-        <v>995</v>
-      </c>
-      <c r="I37" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>1002</v>
+        <v>981</v>
       </c>
       <c r="B38" t="s">
         <v>126</v>
@@ -12640,21 +12499,18 @@
         <v>570</v>
       </c>
       <c r="F38" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="G38" t="s">
-        <v>925</v>
-      </c>
-      <c r="I38" t="s">
-        <v>1003</v>
-      </c>
-      <c r="J38" t="s">
-        <v>1004</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+      <c r="H38" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>1005</v>
+        <v>982</v>
       </c>
       <c r="B39" t="s">
         <v>130</v>
@@ -12669,21 +12525,21 @@
         <v>890</v>
       </c>
       <c r="F39" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="G39" t="s">
-        <v>925</v>
-      </c>
-      <c r="I39" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+        <v>923</v>
+      </c>
+      <c r="H39" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>1006</v>
+        <v>984</v>
       </c>
       <c r="B40" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="C40" t="s">
         <v>506</v>
@@ -12695,24 +12551,21 @@
         <v>505</v>
       </c>
       <c r="F40" t="s">
-        <v>1007</v>
+        <v>983</v>
       </c>
       <c r="G40" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H40" t="s">
-        <v>1008</v>
-      </c>
-      <c r="I40" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>1009</v>
+        <v>985</v>
       </c>
       <c r="B41" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="C41" t="s">
         <v>506</v>
@@ -12724,21 +12577,18 @@
         <v>887</v>
       </c>
       <c r="F41" t="s">
-        <v>1007</v>
+        <v>983</v>
       </c>
       <c r="G41" t="s">
+        <v>927</v>
+      </c>
+      <c r="H41" t="s">
         <v>930</v>
       </c>
-      <c r="H41" t="s">
-        <v>1010</v>
-      </c>
-      <c r="I41" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>1011</v>
+        <v>986</v>
       </c>
       <c r="B42" t="s">
         <v>880</v>
@@ -12753,30 +12603,24 @@
         <v>229</v>
       </c>
       <c r="F42" t="s">
+        <v>947</v>
+      </c>
+      <c r="G42" t="s">
         <v>952</v>
-      </c>
-      <c r="G42" t="s">
-        <v>958</v>
       </c>
       <c r="H42" t="s">
         <v>739</v>
       </c>
-      <c r="I42" t="s">
-        <v>568</v>
-      </c>
-      <c r="J42" t="s">
-        <v>1012</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>1013</v>
+        <v>987</v>
       </c>
       <c r="B43" t="s">
+        <v>900</v>
+      </c>
+      <c r="C43" t="s">
         <v>901</v>
-      </c>
-      <c r="C43" t="s">
-        <v>902</v>
       </c>
       <c r="D43" t="s">
         <v>880</v>
@@ -12785,21 +12629,18 @@
         <v>570</v>
       </c>
       <c r="F43" t="s">
-        <v>1007</v>
+        <v>983</v>
       </c>
       <c r="G43" t="s">
-        <v>930</v>
-      </c>
-      <c r="I43" t="s">
-        <v>568</v>
-      </c>
-      <c r="J43" t="s">
-        <v>1014</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+        <v>927</v>
+      </c>
+      <c r="H43" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>1015</v>
+        <v>988</v>
       </c>
       <c r="B44" t="s">
         <v>133</v>
@@ -12814,21 +12655,18 @@
         <v>581</v>
       </c>
       <c r="F44" t="s">
-        <v>986</v>
+        <v>965</v>
       </c>
       <c r="G44" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H44" t="s">
-        <v>1016</v>
-      </c>
-      <c r="I44" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>1017</v>
+        <v>990</v>
       </c>
       <c r="B45" t="s">
         <v>878</v>
@@ -12837,27 +12675,21 @@
         <v>593</v>
       </c>
       <c r="E45" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="F45" t="s">
-        <v>1018</v>
+        <v>989</v>
       </c>
       <c r="G45" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H45" t="s">
-        <v>1016</v>
-      </c>
-      <c r="I45" t="s">
-        <v>603</v>
-      </c>
-      <c r="J45" t="s">
-        <v>1019</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>1020</v>
+        <v>992</v>
       </c>
       <c r="B46" t="s">
         <v>879</v>
@@ -12866,27 +12698,21 @@
         <v>721</v>
       </c>
       <c r="E46" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="F46" t="s">
-        <v>1021</v>
+        <v>991</v>
       </c>
       <c r="G46" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H46" t="s">
         <v>168</v>
       </c>
-      <c r="I46" t="s">
-        <v>719</v>
-      </c>
-      <c r="J46" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>1023</v>
+        <v>993</v>
       </c>
       <c r="B47" t="s">
         <v>879</v>
@@ -12895,27 +12721,21 @@
         <v>721</v>
       </c>
       <c r="E47" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="F47" t="s">
-        <v>957</v>
+        <v>951</v>
       </c>
       <c r="G47" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H47" t="s">
         <v>498</v>
       </c>
-      <c r="I47" t="s">
-        <v>719</v>
-      </c>
-      <c r="J47" t="s">
-        <v>1024</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>1025</v>
+        <v>994</v>
       </c>
       <c r="B48" t="s">
         <v>104</v>
@@ -12924,24 +12744,18 @@
         <v>105</v>
       </c>
       <c r="E48" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="F48" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G48" t="s">
-        <v>930</v>
-      </c>
-      <c r="H48" t="s">
-        <v>1026</v>
-      </c>
-      <c r="I48" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>1027</v>
+        <v>995</v>
       </c>
       <c r="B49" t="s">
         <v>112</v>
@@ -12956,21 +12770,15 @@
         <v>229</v>
       </c>
       <c r="F49" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G49" t="s">
-        <v>930</v>
-      </c>
-      <c r="H49" t="s">
-        <v>1028</v>
-      </c>
-      <c r="I49" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>1029</v>
+        <v>996</v>
       </c>
       <c r="B50" t="s">
         <v>832</v>
@@ -12985,47 +12793,41 @@
         <v>229</v>
       </c>
       <c r="F50" t="s">
-        <v>1066</v>
+        <v>1029</v>
       </c>
       <c r="G50" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H50" t="s">
-        <v>1030</v>
-      </c>
-      <c r="I50" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>1032</v>
+        <v>997</v>
       </c>
       <c r="C51" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="E51" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="F51" t="s">
+        <v>947</v>
+      </c>
+      <c r="G51" t="s">
         <v>952</v>
-      </c>
-      <c r="G51" t="s">
-        <v>958</v>
       </c>
       <c r="H51" t="s">
         <v>177</v>
       </c>
-      <c r="I51" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>1033</v>
+        <v>998</v>
       </c>
       <c r="C52" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="D52" t="s">
         <v>869</v>
@@ -13034,24 +12836,21 @@
         <v>369</v>
       </c>
       <c r="F52" t="s">
-        <v>957</v>
+        <v>951</v>
       </c>
       <c r="G52" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H52" t="s">
         <v>168</v>
       </c>
-      <c r="I52" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>1034</v>
+        <v>1000</v>
       </c>
       <c r="C53" t="s">
-        <v>1035</v>
+        <v>999</v>
       </c>
       <c r="D53" t="s">
         <v>856</v>
@@ -13060,24 +12859,21 @@
         <v>267</v>
       </c>
       <c r="F53" t="s">
-        <v>998</v>
+        <v>976</v>
       </c>
       <c r="G53" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H53" t="s">
         <v>184</v>
       </c>
-      <c r="I53" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>1036</v>
+        <v>1002</v>
       </c>
       <c r="C54" t="s">
-        <v>1037</v>
+        <v>1001</v>
       </c>
       <c r="D54" t="s">
         <v>850</v>
@@ -13086,21 +12882,18 @@
         <v>229</v>
       </c>
       <c r="F54" t="s">
+        <v>947</v>
+      </c>
+      <c r="G54" t="s">
         <v>952</v>
-      </c>
-      <c r="G54" t="s">
-        <v>958</v>
       </c>
       <c r="H54" t="s">
         <v>168</v>
       </c>
-      <c r="I54" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>1038</v>
+        <v>1003</v>
       </c>
       <c r="B55" t="s">
         <v>889</v>
@@ -13115,24 +12908,21 @@
         <v>229</v>
       </c>
       <c r="F55" t="s">
+        <v>947</v>
+      </c>
+      <c r="G55" t="s">
         <v>952</v>
-      </c>
-      <c r="G55" t="s">
-        <v>958</v>
       </c>
       <c r="H55" t="s">
         <v>168</v>
       </c>
-      <c r="I55" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>1039</v>
+        <v>1005</v>
       </c>
       <c r="C56" t="s">
-        <v>1040</v>
+        <v>1004</v>
       </c>
       <c r="D56" t="s">
         <v>850</v>
@@ -13141,21 +12931,18 @@
         <v>229</v>
       </c>
       <c r="F56" t="s">
+        <v>947</v>
+      </c>
+      <c r="G56" t="s">
         <v>952</v>
-      </c>
-      <c r="G56" t="s">
-        <v>958</v>
       </c>
       <c r="H56" t="s">
         <v>168</v>
       </c>
-      <c r="I56" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>1041</v>
+        <v>1006</v>
       </c>
       <c r="B57" t="s">
         <v>886</v>
@@ -13170,47 +12957,41 @@
         <v>229</v>
       </c>
       <c r="F57" t="s">
+        <v>947</v>
+      </c>
+      <c r="G57" t="s">
         <v>952</v>
-      </c>
-      <c r="G57" t="s">
-        <v>958</v>
       </c>
       <c r="H57" t="s">
         <v>215</v>
       </c>
-      <c r="I57" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>1042</v>
+        <v>1008</v>
       </c>
       <c r="C58" t="s">
-        <v>1040</v>
+        <v>1004</v>
       </c>
       <c r="E58" t="s">
-        <v>1043</v>
+        <v>1007</v>
       </c>
       <c r="F58" t="s">
-        <v>957</v>
+        <v>951</v>
       </c>
       <c r="G58" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H58" t="s">
-        <v>995</v>
-      </c>
-      <c r="I58" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>1044</v>
+        <v>1011</v>
       </c>
       <c r="C59" t="s">
-        <v>1045</v>
+        <v>1009</v>
       </c>
       <c r="D59" t="s">
         <v>850</v>
@@ -13219,24 +13000,21 @@
         <v>229</v>
       </c>
       <c r="F59" t="s">
+        <v>947</v>
+      </c>
+      <c r="G59" t="s">
         <v>952</v>
       </c>
-      <c r="G59" t="s">
-        <v>958</v>
-      </c>
       <c r="H59" t="s">
-        <v>1046</v>
-      </c>
-      <c r="I59" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>1047</v>
+        <v>1014</v>
       </c>
       <c r="C60" t="s">
-        <v>1048</v>
+        <v>1012</v>
       </c>
       <c r="D60" t="s">
         <v>850</v>
@@ -13245,21 +13023,18 @@
         <v>229</v>
       </c>
       <c r="F60" t="s">
+        <v>947</v>
+      </c>
+      <c r="G60" t="s">
         <v>952</v>
       </c>
-      <c r="G60" t="s">
-        <v>958</v>
-      </c>
       <c r="H60" t="s">
-        <v>1049</v>
-      </c>
-      <c r="I60" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>1050</v>
+        <v>1017</v>
       </c>
       <c r="B61" t="s">
         <v>850</v>
@@ -13268,24 +13043,21 @@
         <v>229</v>
       </c>
       <c r="E61" t="s">
-        <v>1051</v>
+        <v>1015</v>
       </c>
       <c r="F61" t="s">
-        <v>998</v>
+        <v>976</v>
       </c>
       <c r="G61" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H61" t="s">
-        <v>1052</v>
-      </c>
-      <c r="I61" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>1053</v>
+        <v>1018</v>
       </c>
       <c r="B62" t="s">
         <v>85</v>
@@ -13300,21 +13072,18 @@
         <v>867</v>
       </c>
       <c r="F62" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="G62" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H62" t="s">
-        <v>184</v>
-      </c>
-      <c r="I62" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>1054</v>
+        <v>1019</v>
       </c>
       <c r="B63" t="s">
         <v>874</v>
@@ -13329,24 +13098,21 @@
         <v>867</v>
       </c>
       <c r="F63" t="s">
-        <v>998</v>
+        <v>976</v>
       </c>
       <c r="G63" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H63" t="s">
         <v>184</v>
       </c>
-      <c r="I63" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>1055</v>
+        <v>1021</v>
       </c>
       <c r="C64" t="s">
-        <v>1056</v>
+        <v>1020</v>
       </c>
       <c r="D64" t="s">
         <v>874</v>
@@ -13355,21 +13121,18 @@
         <v>298</v>
       </c>
       <c r="F64" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G64" t="s">
-        <v>930</v>
-      </c>
-      <c r="I64" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>1057</v>
+        <v>1023</v>
       </c>
       <c r="C65" t="s">
-        <v>1058</v>
+        <v>1022</v>
       </c>
       <c r="D65" t="s">
         <v>874</v>
@@ -13378,21 +13141,18 @@
         <v>298</v>
       </c>
       <c r="F65" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G65" t="s">
-        <v>930</v>
-      </c>
-      <c r="I65" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>1059</v>
+        <v>1025</v>
       </c>
       <c r="C66" t="s">
-        <v>1060</v>
+        <v>1024</v>
       </c>
       <c r="D66" t="s">
         <v>874</v>
@@ -13401,21 +13161,18 @@
         <v>298</v>
       </c>
       <c r="F66" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="G66" t="s">
-        <v>930</v>
-      </c>
-      <c r="I66" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>1061</v>
+        <v>1027</v>
       </c>
       <c r="C67" t="s">
-        <v>1062</v>
+        <v>1026</v>
       </c>
       <c r="D67" t="s">
         <v>866</v>
@@ -13424,21 +13181,18 @@
         <v>867</v>
       </c>
       <c r="F67" t="s">
-        <v>1007</v>
+        <v>983</v>
       </c>
       <c r="G67" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="H67" t="s">
-        <v>1063</v>
-      </c>
-      <c r="I67" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>1064</v>
+        <v>1030</v>
       </c>
       <c r="B68" t="s">
         <v>866</v>
@@ -13447,24 +13201,21 @@
         <v>867</v>
       </c>
       <c r="E68" t="s">
-        <v>1065</v>
+        <v>1028</v>
       </c>
       <c r="F68" t="s">
-        <v>998</v>
+        <v>976</v>
       </c>
       <c r="G68" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="H68" t="s">
-        <v>995</v>
-      </c>
-      <c r="I68" t="s">
-        <v>1031</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>1067</v>
+        <v>1040</v>
       </c>
       <c r="B69" t="s">
         <v>844</v>
@@ -13479,13 +13230,13 @@
         <v>229</v>
       </c>
       <c r="F69" t="s">
-        <v>1068</v>
+        <v>1031</v>
       </c>
       <c r="G69" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="H69" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dati: Persone ~1, Relazioni +2
Persone — modificati: AMI-P-007
Relazioni — aggiunti: AMI-R-070, AMI-R-071
Altri file: Launcher.py, README.md, documentazione, mkdocs.yml, assets
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50390168-6F12-4919-B523-A308F8F83507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00CFD43-FB2B-448F-AE27-357FA06C7482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2706" uniqueCount="1067">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2723" uniqueCount="1071">
   <si>
     <t>ID_relazione</t>
   </si>
@@ -3302,12 +3302,24 @@
   <si>
     <t>1967-1969</t>
   </si>
+  <si>
+    <t>AMI-R-070</t>
+  </si>
+  <si>
+    <t>1972-1977</t>
+  </si>
+  <si>
+    <t>AMI-R-071</t>
+  </si>
+  <si>
+    <t>dino-dini.png</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3335,6 +3347,12 @@
       <color theme="1"/>
       <name val="Georgia"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -9588,6 +9606,9 @@
       <c r="I8" t="s">
         <v>942</v>
       </c>
+      <c r="J8" t="s">
+        <v>1070</v>
+      </c>
       <c r="O8" t="s">
         <v>925</v>
       </c>
@@ -11681,7 +11702,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
@@ -13377,7 +13398,60 @@
         <v>15</v>
       </c>
     </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B70" t="s">
+        <v>107</v>
+      </c>
+      <c r="C70" t="s">
+        <v>108</v>
+      </c>
+      <c r="D70" t="s">
+        <v>104</v>
+      </c>
+      <c r="E70" t="s">
+        <v>105</v>
+      </c>
+      <c r="F70" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" t="s">
+        <v>14</v>
+      </c>
+      <c r="H70" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B71" t="s">
+        <v>217</v>
+      </c>
+      <c r="C71" t="s">
+        <v>218</v>
+      </c>
+      <c r="D71" t="s">
+        <v>11</v>
+      </c>
+      <c r="E71" t="s">
+        <v>12</v>
+      </c>
+      <c r="F71" t="s">
+        <v>19</v>
+      </c>
+      <c r="G71" t="s">
+        <v>20</v>
+      </c>
+      <c r="H71" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Dati: Organizzazioni ~1 (AMI-O-022)
Organizzazioni — modificati: AMI-O-022
Altri file: assets
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC73B3D-7387-4037-8C05-23CC62F14CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC8135C5-AAF0-4479-9100-CED900110887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2723" uniqueCount="1071">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2724" uniqueCount="1072">
   <si>
     <t>ID_relazione</t>
   </si>
@@ -3313,6 +3313,9 @@
   </si>
   <si>
     <t>PC(m-l-m)I</t>
+  </si>
+  <si>
+    <t>Circolo Lenin di Budrio; Circolo Lenin di Faenza; Circoli Lenin di Budrio, Bologna e Castenaso</t>
   </si>
 </sst>
 </file>
@@ -11397,6 +11400,9 @@
       <c r="E23" t="s">
         <v>171</v>
       </c>
+      <c r="F23" t="s">
+        <v>1071</v>
+      </c>
       <c r="G23" t="s">
         <v>1039</v>
       </c>

</xml_diff>

<commit_message>
Dati: Organizzazioni ~1 (AMI-O-006)
Organizzazioni — modificati: AMI-O-006
Altri file: DESIGN.md, assets, documentazione, scripts
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC8135C5-AAF0-4479-9100-CED900110887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71EFCEA6-CEB7-4FA5-B71C-62A0BACB7EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2724" uniqueCount="1072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2725" uniqueCount="1073">
   <si>
     <t>ID_relazione</t>
   </si>
@@ -3316,6 +3316,9 @@
   </si>
   <si>
     <t>Circolo Lenin di Budrio; Circolo Lenin di Faenza; Circoli Lenin di Budrio, Bologna e Castenaso</t>
+  </si>
+  <si>
+    <t>Per la vittoria del marxismo-leninismo; Organo del Movimento Marxista-Leninista Italiano; Organo centrale del Partito Comunista d’Italia (m-l)</t>
   </si>
 </sst>
 </file>
@@ -3404,6 +3407,21 @@
   </cellStyles>
   <dxfs count="7">
     <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
@@ -3430,21 +3448,6 @@
         <sz val="11"/>
         <color theme="0"/>
         <name val="Calibri"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
       </font>
     </dxf>
   </dxfs>
@@ -3492,13 +3495,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabella6" displayName="Tabella6" ref="A1:D23" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabella6" displayName="Tabella6" ref="A1:D23" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A1:D23" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Codice_ISAD" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Elemento" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Valore" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Note" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Codice_ISAD" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Elemento" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Valore" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Note" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3559,7 +3562,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabella5" displayName="Tabella5" ref="A1:H84" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabella5" displayName="Tabella5" ref="A1:H84" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:H84" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="ID_relazione"/>
@@ -10729,6 +10732,9 @@
       <c r="E7" t="s">
         <v>192</v>
       </c>
+      <c r="F7" t="s">
+        <v>1072</v>
+      </c>
       <c r="G7" t="s">
         <v>1027</v>
       </c>

</xml_diff>

<commit_message>
Dati: Catalogo +1 ~1 (AMI-0110, AMI-0109)
Catalogo — aggiunti: AMI-0110
Catalogo — modificati: AMI-0109
Altri file: scripts
</commit_message>
<xml_diff>
--- a/data/dati.xlsx
+++ b/data/dati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5651B5-F346-42C2-A111-C9AA04AEDFF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46DB9F3-78BF-4978-A256-66EEC3AED0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogo" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2962" uniqueCount="1150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2974" uniqueCount="1152">
   <si>
     <t>ID_relazione</t>
   </si>
@@ -3546,10 +3546,16 @@
     <t>https://archive.org/details/1985-documenti-del-iv-congresso/mode/2up</t>
   </si>
   <si>
-    <t>s.l.</t>
-  </si>
-  <si>
     <t>Nuova Unità; Unione della Gioventù Comunista d'Italia (marxista-leninista)</t>
+  </si>
+  <si>
+    <t>AMI-0110</t>
+  </si>
+  <si>
+    <t>La forza di essere comunisti: Che cosa vuole il Partito Comunista d'Italia (m-l)</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/la-forza-di-essere-comunisti/mode/2up</t>
   </si>
 </sst>
 </file>
@@ -4847,7 +4853,7 @@
         <v>329</v>
       </c>
       <c r="O14" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="P14" t="s">
         <v>270</v>
@@ -9775,9 +9781,6 @@
       <c r="K110" t="s">
         <v>274</v>
       </c>
-      <c r="L110" t="s">
-        <v>1148</v>
-      </c>
       <c r="M110" t="s">
         <v>328</v>
       </c>
@@ -9792,7 +9795,51 @@
       </c>
     </row>
     <row r="111" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="Q111" s="3"/>
+      <c r="A111" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B111" t="s">
+        <v>262</v>
+      </c>
+      <c r="C111" t="s">
+        <v>263</v>
+      </c>
+      <c r="D111" t="s">
+        <v>1150</v>
+      </c>
+      <c r="E111" t="s">
+        <v>265</v>
+      </c>
+      <c r="F111" t="s">
+        <v>12</v>
+      </c>
+      <c r="G111" t="s">
+        <v>10</v>
+      </c>
+      <c r="H111" t="s">
+        <v>1144</v>
+      </c>
+      <c r="I111">
+        <v>1986</v>
+      </c>
+      <c r="J111">
+        <v>1986</v>
+      </c>
+      <c r="K111" t="s">
+        <v>267</v>
+      </c>
+      <c r="L111" t="s">
+        <v>812</v>
+      </c>
+      <c r="M111" t="s">
+        <v>328</v>
+      </c>
+      <c r="P111" t="s">
+        <v>1080</v>
+      </c>
+      <c r="Q111" s="3" t="s">
+        <v>1151</v>
+      </c>
     </row>
     <row r="112" spans="1:22" x14ac:dyDescent="0.3">
       <c r="Q112" s="3"/>
@@ -10037,11 +10084,12 @@
     <hyperlink ref="Q105" r:id="rId107" xr:uid="{09B963F9-4F3D-4F82-A0E7-92B1358B3997}"/>
     <hyperlink ref="Q109" r:id="rId108" xr:uid="{DA33DC8F-848A-4B19-9DAB-DA96FA1F78B2}"/>
     <hyperlink ref="Q110" r:id="rId109" xr:uid="{54B8C84E-0C88-4EAD-825F-BFEFB5391A5A}"/>
+    <hyperlink ref="Q111" r:id="rId110" xr:uid="{987D79B4-DA9A-4321-BE42-93DC7C7ABA59}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId110"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId111"/>
   <tableParts count="1">
-    <tablePart r:id="rId111"/>
+    <tablePart r:id="rId112"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>